<commit_message>
fix(auditoria): corrigir auditor, modalidade I6/I7, evidencias de 8.2.3-8.2.6 e visibilidade dos titulos de secao
</commit_message>
<xml_diff>
--- a/FOR.143.r01_Formulário_de_Check_List_da_Auditoria_ISO_13485.xlsx
+++ b/FOR.143.r01_Formulário_de_Check_List_da_Auditoria_ISO_13485.xlsx
@@ -26,7 +26,7 @@
     <numFmt numFmtId="164" formatCode="d\.m"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="38">
+  <fonts count="41">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -239,8 +239,24 @@
       <color rgb="FF000000"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -293,6 +309,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF6B26B"/>
         <bgColor rgb="FFF6B26B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+        <bgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -499,7 +521,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="145">
+  <cellXfs count="149">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -883,6 +905,18 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1261,7 +1295,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="pt-BR"/>
               </a:p>
@@ -1286,7 +1320,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="pt-BR"/>
           </a:p>
@@ -1340,7 +1374,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="pt-BR"/>
               </a:p>
@@ -1370,7 +1404,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="pt-BR"/>
           </a:p>
@@ -1396,7 +1430,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR"/>
         </a:p>
@@ -1754,7 +1788,7 @@
       </c>
       <c r="C6" s="132" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>Vinicius Mota</t>
         </is>
       </c>
       <c r="D6" s="127" t="n"/>
@@ -1762,7 +1796,11 @@
       <c r="F6" s="127" t="n"/>
       <c r="G6" s="127" t="n"/>
       <c r="H6" s="128" t="n"/>
-      <c r="I6" s="9" t="n"/>
+      <c r="I6" s="145" t="inlineStr">
+        <is>
+          <t>   </t>
+        </is>
+      </c>
       <c r="J6" s="10" t="inlineStr">
         <is>
           <t>Remota</t>
@@ -1785,7 +1823,11 @@
       <c r="F7" s="127" t="n"/>
       <c r="G7" s="127" t="n"/>
       <c r="H7" s="128" t="n"/>
-      <c r="I7" s="9" t="n"/>
+      <c r="I7" s="145" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J7" s="10" t="inlineStr">
         <is>
           <t>Presencial</t>
@@ -1917,7 +1959,7 @@
     </row>
     <row r="13" ht="23.25" customHeight="1" s="104">
       <c r="A13" s="7" t="n"/>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B13" s="146" t="inlineStr">
         <is>
           <t>SISTEMA DE GESTÃO DA QUALIDADE</t>
         </is>
@@ -2310,7 +2352,7 @@
     </row>
     <row r="25" ht="23.25" customHeight="1" s="104">
       <c r="A25" s="24" t="n"/>
-      <c r="B25" s="14" t="inlineStr">
+      <c r="B25" s="146" t="inlineStr">
         <is>
           <t>RESPONSABILIDADE DA DIREÇÃO</t>
         </is>
@@ -2714,7 +2756,7 @@
     </row>
     <row r="37" ht="23.25" customHeight="1" s="104">
       <c r="A37" s="24" t="n"/>
-      <c r="B37" s="14" t="inlineStr">
+      <c r="B37" s="146" t="inlineStr">
         <is>
           <t>GESTÃO DE RECURSOS</t>
         </is>
@@ -2969,7 +3011,7 @@
     </row>
     <row r="43" ht="23.25" customHeight="1" s="104">
       <c r="A43" s="24" t="n"/>
-      <c r="B43" s="14" t="inlineStr">
+      <c r="B43" s="146" t="inlineStr">
         <is>
           <t>REALIZAÇÃO DE PRODUTO (FABRICAÇÃO)</t>
         </is>
@@ -3934,7 +3976,7 @@
     </row>
     <row r="74" ht="23.25" customHeight="1" s="104">
       <c r="A74" s="24" t="n"/>
-      <c r="B74" s="14" t="inlineStr">
+      <c r="B74" s="146" t="inlineStr">
         <is>
           <t>MEDIÇÃO, ANÁLISE E MELHORIA</t>
         </is>
@@ -4096,7 +4138,7 @@
           <t>A organização documenta procedimento para notificação às autoridades provenientes de ações relacionadas ao produto? Evento adverso, alterações importantes, recolhimento. Os registros são mantidos conforme item 4.2.5?</t>
         </is>
       </c>
-      <c r="D78" s="28" t="inlineStr">
+      <c r="D78" s="147" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4104,7 +4146,20 @@
       <c r="E78" s="27" t="n"/>
       <c r="F78" s="27" t="n"/>
       <c r="G78" s="27" t="n"/>
-      <c r="H78" s="35" t="n"/>
+      <c r="H78" s="148" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.022.R5: Não Conformidade - Ações Corretivas e Preventivas: A organização deve realizar o acompanhamento de todas as soluções de problemas e oportunidades de melhorias criadas para que o sistema de qualidade esteja em constante melhoria dos seus processos. Neste sentido, é obrigatório inserir todos os registros relacionados no Controle Anual de Registros: Plano de Ação, RNC, 8D, Gestão de Mudança e Revisão Gerencial.
+• [Conforme] POP.1057.R0: Manual Operacional - Comunicação com o Cliente - Visolab: 2. RECLAMAÇÕES: 
+2.1 Recebimento de Reclamações 
+2.2 Tratativa das Reclamações:
+3.DEVOLUTIVAS PARA O CLIENTE:
+As devolutivas aos clientes são enviadas de acordo com o canal utilizado pelo mesmo.
+• [Conforme] POP.1012.R1: Monitoramento de Realimentação do Cliente - Visolab: 2. REGISTRO DAS RECLAMAÇÕES DE CLIENTES:
+2.1 Registro de Realimentação de clientes através do atendimento
+3. ACOMPANHAMENTO DE RETORNOS:
+4. PESQUISA ANUAL DE SATISFAÇÃO</t>
+        </is>
+      </c>
       <c r="I78" s="136" t="n"/>
       <c r="J78" s="128" t="n"/>
       <c r="K78" s="22" t="n"/>
@@ -4123,7 +4178,7 @@
           <t>A organização possui procedimento para auditoria interna? As autoridades são definidas? Os registros são mantidos? É realizado acompanhamento de atividades apontadas em outras auditorias?</t>
         </is>
       </c>
-      <c r="D79" s="28" t="inlineStr">
+      <c r="D79" s="147" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4131,7 +4186,14 @@
       <c r="E79" s="27" t="n"/>
       <c r="F79" s="27" t="n"/>
       <c r="G79" s="27" t="n"/>
-      <c r="H79" s="35" t="n"/>
+      <c r="H79" s="148" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.024.R3: Auditoria: FOR.140: Relatório de Auditoria Interna, 
+FOR.123: Agenda de Auditoria, 
+FOR.167: Cronograma de Auditoria, 
+FOR.143: Formulário de Check List da Auditoria ISO 1348</t>
+        </is>
+      </c>
       <c r="I79" s="35" t="n"/>
       <c r="J79" s="128" t="n"/>
       <c r="K79" s="22" t="n"/>
@@ -4150,7 +4212,7 @@
           <t>É realizado monitoramento e medição dos processos do SGQ? Possui KPIs? Os resultados planejados que não forem alcançados, são realizadas correções e ações corretivas?</t>
         </is>
       </c>
-      <c r="D80" s="28" t="inlineStr">
+      <c r="D80" s="147" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4158,7 +4220,12 @@
       <c r="E80" s="27" t="n"/>
       <c r="F80" s="27" t="n"/>
       <c r="G80" s="27" t="n"/>
-      <c r="H80" s="35" t="n"/>
+      <c r="H80" s="148" t="inlineStr">
+        <is>
+          <t>• [Conforme] Evidências / Documentos Registrados: MAQ.002.R10 - Manual da Qualidade:
+- Objetivos da Qualidade</t>
+        </is>
+      </c>
       <c r="I80" s="35" t="n"/>
       <c r="J80" s="128" t="n"/>
       <c r="K80" s="22" t="n"/>
@@ -4177,7 +4244,7 @@
           <t xml:space="preserve">A organização monitora características e requisitos do produto? É realizado registro dos responsáveis por liberação do produto para fim de rastreabilidade? </t>
         </is>
       </c>
-      <c r="D81" s="28" t="inlineStr">
+      <c r="D81" s="147" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4185,7 +4252,25 @@
       <c r="E81" s="27" t="n"/>
       <c r="F81" s="27" t="n"/>
       <c r="G81" s="27" t="n"/>
-      <c r="H81" s="35" t="n"/>
+      <c r="H81" s="148" t="inlineStr">
+        <is>
+          <t>• [Conforme] Evidências / Documentos Registrados: PSQ.018.R2 - Realização de Produto; 
+PSQ.017.R3 - Controle de Documentos e Registros; 
+PSQ.019.R2 - Preservação de Insumo e Produto; 
+PSQ.022.R5 - Não Conformidade -Ações Corretivas e Preventivas; 
+PSQ.023.R4 - Treinamentos; 
+PSQ.024.R3 - Auditoria; 
+PSQ.026.R1 - Identificação e Rastreabilidade; 
+PSQ.027.R2 - Validação; 
+PSQ.028.R5 - Gestão de Risco; 
+PSQ.029.R3 - Gestão de Mudança; 
+PSQ.031.R0 - Gerenciamento de Claim de Produtos e Serviços; 
+PSQ.032.R7 - Monitoramento de Equipamento de Medição; 
+PSQ.033.R2 - Manutenção; 
+PSQ.025.R1 - Revisão Gerencial; 
+POP.1002.R1 - Manual Operacional - Rastreabilidade de Pedidos Visolab</t>
+        </is>
+      </c>
       <c r="I81" s="35" t="n"/>
       <c r="J81" s="128" t="n"/>
       <c r="K81" s="22" t="n"/>

</xml_diff>

<commit_message>
fix(checklist): remover linhas extras de agrupadores pai e restaurar estrutura original do template
</commit_message>
<xml_diff>
--- a/FOR.143.r01_Formulário_de_Check_List_da_Auditoria_ISO_13485.xlsx
+++ b/FOR.143.r01_Formulário_de_Check_List_da_Auditoria_ISO_13485.xlsx
@@ -26,7 +26,7 @@
     <numFmt numFmtId="164" formatCode="d\.m"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="41">
+  <fonts count="40">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -238,12 +238,6 @@
       <b val="1"/>
       <color rgb="FF000000"/>
       <sz val="8"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -568,7 +562,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="160">
+  <cellXfs count="157">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -931,8 +925,29 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="38" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="10" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="38" fillId="10" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="38" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -952,43 +967,15 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="10" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="39" fillId="10" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="39" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1743,7 +1730,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N94"/>
+  <dimension ref="A1:M94"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.5546875" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="1.109375" customWidth="1" style="104" min="1" max="1"/>
@@ -1868,7 +1855,7 @@
       <c r="F6" s="127" t="n"/>
       <c r="G6" s="127" t="n"/>
       <c r="H6" s="128" t="n"/>
-      <c r="I6" s="149" t="inlineStr">
+      <c r="I6" s="9" t="inlineStr">
         <is>
           <t>   </t>
         </is>
@@ -1889,13 +1876,17 @@
           <t>Data de Auditoria:</t>
         </is>
       </c>
-      <c r="C7" s="133" t="n"/>
+      <c r="C7" s="133" t="inlineStr">
+        <is>
+          <t>20/05/2026 a 22/07/2026</t>
+        </is>
+      </c>
       <c r="D7" s="127" t="n"/>
       <c r="E7" s="127" t="n"/>
       <c r="F7" s="127" t="n"/>
       <c r="G7" s="127" t="n"/>
       <c r="H7" s="128" t="n"/>
-      <c r="I7" s="149" t="inlineStr">
+      <c r="I7" s="9" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -1918,7 +1909,7 @@
       </c>
       <c r="C8" s="132" t="inlineStr">
         <is>
-          <t>Aplicação de antirreflexo (Crizal Rock, Sapphire HR, Optifog e Prevencia), Surfaçagem Digital (Varilux Sport, Varilux Sport Wrap, Varilux Roadpilot, Stellest e Varilux XR 1.74 e Varilux XR cil maior que -4).</t>
+          <t>Laboratório de Montagem e Distribuição de Lentes Oftálmicas</t>
         </is>
       </c>
       <c r="D8" s="127" t="n"/>
@@ -2031,7 +2022,7 @@
     </row>
     <row r="13" ht="23.25" customHeight="1" s="104">
       <c r="A13" s="7" t="n"/>
-      <c r="B13" s="146" t="inlineStr">
+      <c r="B13" s="136" t="inlineStr">
         <is>
           <t>SISTEMA DE GESTÃO DA QUALIDADE</t>
         </is>
@@ -2057,7 +2048,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="62.25" customHeight="1" s="104">
+    <row r="14" ht="48" customHeight="1" s="104">
       <c r="A14" s="16" t="n"/>
       <c r="B14" s="17" t="inlineStr">
         <is>
@@ -2069,22 +2060,22 @@
           <t>A organização documenta seu papel em relação aos requisitos regulatórios aplicáveis?</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="D14" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
-      <c r="H14" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Manual de compras: DOC.085.R0 - Manual de Compras - Visolab
-• [Conforme] Procedimento para recebimento de lentes e bloco: POP.1122.R0: Manual Operacional - Armazenamento de blocos e lentes no estoque
-• [Conforme] MAQ.002.R10: Manual da Qualidade: PSQ.033.R2: Procedimento de Manutenção</t>
-        </is>
-      </c>
-      <c r="I14" s="19" t="n"/>
+      <c r="E14" s="154" t="n"/>
+      <c r="F14" s="154" t="n"/>
+      <c r="G14" s="154" t="n"/>
+      <c r="H14" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] Manual de compras: DOC.085.R0  Manual de Compras - Visolab
+• [Conforme] Procedimento para recebimento de lentes e bloco: POP.1122.R0: Manual Operacional - Recebimento de Lentes e Blocos - Visolab
+• [Conforme] Gestão de Riscos: PSQ.028.R5: Gestão de Risco</t>
+        </is>
+      </c>
+      <c r="I14" s="142" t="n"/>
       <c r="J14" s="128" t="n"/>
       <c r="K14" s="20">
         <f>(K13)/(K13+L13+M13)</f>
@@ -2099,7 +2090,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="55.2" customHeight="1" s="104">
+    <row r="15" ht="96" customHeight="1" s="104">
       <c r="A15" s="16" t="n"/>
       <c r="B15" s="17" t="inlineStr">
         <is>
@@ -2114,29 +2105,31 @@
 - Sequência e  intereção dos processos.</t>
         </is>
       </c>
-      <c r="D15" s="21" t="inlineStr">
+      <c r="D15" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
-      <c r="H15" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: MAQ.002: Manual da Qualidade
-4.2Requisitos de documentação: 
-4.2.1 Geral: 
-A  estrutura  da  Documentação  do  QMS  daEssilorLuxotticaobedece  a  umahierarquia  dividida  em níveis, conforme (Tab.03)</t>
-        </is>
-      </c>
-      <c r="I15" s="19" t="n"/>
+      <c r="E15" s="154" t="n"/>
+      <c r="F15" s="154" t="n"/>
+      <c r="G15" s="154" t="n"/>
+      <c r="H15" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] MAQ.002.R10 - Manual da Qualidade:
+- Organograma
+- Gestão de Risco
+- Interação de Processos
+- Tabela de Competência e Responsabilidade
+• [Conforme] Matriz de Risco do SGQ e Processos: FOR.061: Matriz de Risco Geral</t>
+        </is>
+      </c>
+      <c r="I15" s="142" t="n"/>
       <c r="J15" s="128" t="n"/>
       <c r="K15" s="22" t="n"/>
       <c r="L15" s="22" t="n"/>
       <c r="M15" s="22" t="n"/>
     </row>
-    <row r="16" ht="62.25" customHeight="1" s="104">
+    <row r="16" ht="20" customHeight="1" s="104">
       <c r="A16" s="16" t="n"/>
       <c r="B16" s="17" t="inlineStr">
         <is>
@@ -2148,28 +2141,26 @@
           <t>A organização controla a documentação da qualidade? Assegura que a documentação de suporte necessária esteja disponível?</t>
         </is>
       </c>
-      <c r="D16" s="21" t="inlineStr">
+      <c r="D16" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
-      <c r="H16" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: MAQ.002: Manual da Qualidade:
-4.2.4 Controle de documentos:
-Procedimento específico, que, prevê que os documentos do QMS são adequadamente controlados quanto: Metodologia para alterações atuais, responsabilidades e métodos para aprovação, metodologia dedistribuição de versões em locais de uso, métodos para validação dosdocumentos e dados, marcação adequada em casos de retenção, bem como cuidados para manutenção no que tange a legibilidade e identificação.Preferencialmente,os  documentos  são  criados  de  forma  que  qualquer  unidade  da EssilorLuxottica possa utiliza-los, desde que possua o mesmo maquinário / equipamento envolvido. Nos casos  muito  específicos  devido  sistemas  operacionais  distintos  ou controle  e alinhamento  diferenciado com  clientes,  é  possível  criar  um  procedimento  padronizado  para  cada  unidade,  desde  que  o  mesmo respeite a hierarquia de documentos e seja controlado.</t>
-        </is>
-      </c>
-      <c r="I16" s="19" t="n"/>
+      <c r="E16" s="154" t="n"/>
+      <c r="F16" s="154" t="n"/>
+      <c r="G16" s="154" t="n"/>
+      <c r="H16" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] Matriz de Risco do SGQ e Processos: FOR.061: Matriz de Risco Geral</t>
+        </is>
+      </c>
+      <c r="I16" s="142" t="n"/>
       <c r="J16" s="128" t="n"/>
       <c r="K16" s="22" t="n"/>
       <c r="L16" s="22" t="n"/>
       <c r="M16" s="22" t="n"/>
     </row>
-    <row r="17" ht="62.25" customHeight="1" s="104">
+    <row r="17" ht="20" customHeight="1" s="104">
       <c r="A17" s="16" t="n"/>
       <c r="B17" s="17" t="inlineStr">
         <is>
@@ -2181,27 +2172,26 @@
           <t>As mudanças realizadas na documentação são avaliadas com relação ao seu impacto no SGQ e produtos?</t>
         </is>
       </c>
-      <c r="D17" s="21" t="n"/>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="D17" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="10" t="n"/>
-      <c r="H17" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Procedimento de Controle de Documentos e Registros: PSQ.017.R3 - Controle de Documentos e Registros
-• [Não Conforme] Acordo de Qualidade para terceirizado: Foi identificado que não há um acordo de qualidade escrito para o serviço terceirizado na LabRio</t>
-        </is>
-      </c>
-      <c r="I17" s="19" t="n"/>
+      <c r="E17" s="154" t="n"/>
+      <c r="F17" s="154" t="n"/>
+      <c r="G17" s="154" t="n"/>
+      <c r="H17" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.029.R3: Gestão de Mudança: FOR.071: Solicitação de Mudança - SM</t>
+        </is>
+      </c>
+      <c r="I17" s="142" t="n"/>
       <c r="J17" s="128" t="n"/>
       <c r="K17" s="22" t="n"/>
       <c r="L17" s="22" t="n"/>
       <c r="M17" s="22" t="n"/>
     </row>
-    <row r="18" ht="62.25" customHeight="1" s="104">
+    <row r="18" ht="32" customHeight="1" s="104">
       <c r="A18" s="16" t="n"/>
       <c r="B18" s="17" t="inlineStr">
         <is>
@@ -2213,26 +2203,27 @@
           <t>A organização terceiriza algum processo? Monitora e assegura os controles dos processos?</t>
         </is>
       </c>
-      <c r="D18" s="21" t="inlineStr">
+      <c r="D18" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
-      <c r="H18" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: PSQ.020: Gestão de Fornecedores</t>
-        </is>
-      </c>
-      <c r="I18" s="19" t="n"/>
+      <c r="E18" s="154" t="n"/>
+      <c r="F18" s="154" t="n"/>
+      <c r="G18" s="154" t="n"/>
+      <c r="H18" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.018.R2: Realização de Produto: FOR.146: Lista de Fornecedores Qualificados
+• [Conforme] PSQ.018.R2: Realização de Produto: FOR.147: Avaliação e Reavaliação de Fornecedores</t>
+        </is>
+      </c>
+      <c r="I18" s="142" t="n"/>
       <c r="J18" s="128" t="n"/>
       <c r="K18" s="22" t="n"/>
       <c r="L18" s="22" t="n"/>
       <c r="M18" s="22" t="n"/>
     </row>
-    <row r="19" ht="27.6" customHeight="1" s="104">
+    <row r="19" ht="32" customHeight="1" s="104">
       <c r="A19" s="16" t="n"/>
       <c r="B19" s="17" t="inlineStr">
         <is>
@@ -2244,26 +2235,27 @@
           <t>A organização documentou procedimento de validação de softwares que impactem no SGQ?</t>
         </is>
       </c>
-      <c r="D19" s="21" t="inlineStr">
+      <c r="D19" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E19" s="10" t="n"/>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="10" t="n"/>
-      <c r="H19" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Validação de Softwares (Opticlick, Qualiex, Engman e SGO): FOR.159.R1: Validação de Software fornecido para cada software solicitado.</t>
-        </is>
-      </c>
-      <c r="I19" s="19" t="n"/>
+      <c r="E19" s="154" t="n"/>
+      <c r="F19" s="154" t="n"/>
+      <c r="G19" s="154" t="n"/>
+      <c r="H19" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.027.R2: Validação: FOR.166: Validação de Software: 
+Validação do Sistema Sysprola</t>
+        </is>
+      </c>
+      <c r="I19" s="142" t="n"/>
       <c r="J19" s="128" t="n"/>
       <c r="K19" s="22" t="n"/>
       <c r="L19" s="22" t="n"/>
       <c r="M19" s="22" t="n"/>
     </row>
-    <row r="20" ht="62.25" customHeight="1" s="104">
+    <row r="20" ht="32" customHeight="1" s="104">
       <c r="A20" s="16" t="n"/>
       <c r="B20" s="17" t="inlineStr">
         <is>
@@ -2275,29 +2267,27 @@
           <t>A organização documentou a Política da Qualidade?</t>
         </is>
       </c>
-      <c r="D20" s="21" t="inlineStr">
+      <c r="D20" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
-      <c r="H20" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: DOC.032.R1: Política da Qualidade:
-• Aumentar a Satisfação do Cliente e do Consumidor
-• Impulsionar a Conformidade de Nossos Produtos e Serviços
-• Esforçar-se  para entregar nosso compromisso</t>
-        </is>
-      </c>
-      <c r="I20" s="19" t="n"/>
+      <c r="E20" s="154" t="n"/>
+      <c r="F20" s="154" t="n"/>
+      <c r="G20" s="154" t="n"/>
+      <c r="H20" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] MAQ.002.R10 - Manual da Qualidade:
+- Política da Qualidade</t>
+        </is>
+      </c>
+      <c r="I20" s="142" t="n"/>
       <c r="J20" s="128" t="n"/>
       <c r="K20" s="22" t="n"/>
       <c r="L20" s="22" t="n"/>
       <c r="M20" s="22" t="n"/>
     </row>
-    <row r="21" ht="62.25" customHeight="1" s="104">
+    <row r="21" ht="64" customHeight="1" s="104">
       <c r="A21" s="16" t="n"/>
       <c r="B21" s="17" t="inlineStr">
         <is>
@@ -2309,26 +2299,29 @@
           <t>A organização documentou o Manual da Qualidade?</t>
         </is>
       </c>
-      <c r="D21" s="21" t="inlineStr">
+      <c r="D21" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E21" s="23" t="n"/>
-      <c r="F21" s="23" t="n"/>
-      <c r="G21" s="23" t="n"/>
-      <c r="H21" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: MAQ.002.R10: Manual da Qualidade</t>
-        </is>
-      </c>
-      <c r="I21" s="19" t="n"/>
+      <c r="E21" s="154" t="n"/>
+      <c r="F21" s="154" t="n"/>
+      <c r="G21" s="154" t="n"/>
+      <c r="H21" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] MAQ.002.R10 - Manual da Qualidade:
+- Escopo do SGQ
+- Estrutura Organizacional
+- Interação de Processos</t>
+        </is>
+      </c>
+      <c r="I21" s="142" t="n"/>
       <c r="J21" s="128" t="n"/>
       <c r="K21" s="22" t="n"/>
       <c r="L21" s="22" t="n"/>
       <c r="M21" s="22" t="n"/>
     </row>
-    <row r="22" ht="62.25" customHeight="1" s="104">
+    <row r="22" ht="32" customHeight="1" s="104">
       <c r="A22" s="24" t="n"/>
       <c r="B22" s="17" t="inlineStr">
         <is>
@@ -2340,32 +2333,27 @@
           <t>A organização possui documentação dos produtos? (Descrição, especificações, registro, procedimentos relacionados ao produto?)</t>
         </is>
       </c>
-      <c r="D22" s="21" t="inlineStr">
+      <c r="D22" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E22" s="23" t="n"/>
-      <c r="F22" s="23" t="n"/>
-      <c r="G22" s="23" t="n"/>
-      <c r="H22" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: MAQ.002.R10: Manual da Qualidade,
-PSQ.018.R2: Realização de Produto e 
-PSQ.026.R1: Identificação e Rastreabilidade</t>
-        </is>
-      </c>
-      <c r="I22" s="19" t="inlineStr">
-        <is>
-          <t>[OBS com Correção] Disponibilizar para os postos de conferência.</t>
-        </is>
-      </c>
+      <c r="E22" s="154" t="n"/>
+      <c r="F22" s="154" t="n"/>
+      <c r="G22" s="154" t="n"/>
+      <c r="H22" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] POP.1002.R1 - Manual Operacional - Rastreabilidade de Pedidos Visolab
+• [Conforme] DMR: DOC.085.R0  Manual de Compras - Visolab; POP.1057.R0 Manual Operacional - Comunicação com o Cliente - Visolab</t>
+        </is>
+      </c>
+      <c r="I22" s="142" t="n"/>
       <c r="J22" s="128" t="n"/>
       <c r="K22" s="22" t="n"/>
       <c r="L22" s="22" t="n"/>
       <c r="M22" s="22" t="n"/>
     </row>
-    <row r="23" ht="69" customHeight="1" s="104">
+    <row r="23" ht="20" customHeight="1" s="104">
       <c r="A23" s="24" t="n"/>
       <c r="B23" s="17" t="inlineStr">
         <is>
@@ -2377,18 +2365,26 @@
           <t>A organização documentou procedimento para controlar, analisar, aprovar, previnir deterioração, previnir uso não intencional e assegurar que as versões vigentes dos documentos estejam disponíveis?</t>
         </is>
       </c>
-      <c r="D23" s="21" t="n"/>
-      <c r="E23" s="23" t="n"/>
-      <c r="F23" s="23" t="n"/>
-      <c r="G23" s="23" t="n"/>
-      <c r="H23" s="19" t="n"/>
-      <c r="I23" s="19" t="n"/>
+      <c r="D23" s="154" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E23" s="154" t="n"/>
+      <c r="F23" s="154" t="n"/>
+      <c r="G23" s="154" t="n"/>
+      <c r="H23" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.017.R3 - Controle de Documentos e Registros</t>
+        </is>
+      </c>
+      <c r="I23" s="142" t="n"/>
       <c r="J23" s="128" t="n"/>
       <c r="K23" s="22" t="n"/>
       <c r="L23" s="22" t="n"/>
       <c r="M23" s="22" t="n"/>
     </row>
-    <row r="24" ht="62.25" customHeight="1" s="104">
+    <row r="24" ht="20" customHeight="1" s="104">
       <c r="A24" s="24" t="n"/>
       <c r="B24" s="17" t="inlineStr">
         <is>
@@ -2400,23 +2396,20 @@
           <t>A organização documentou procedimento para definir, identificar, armazenar, dar tempo de retenção, garantir a integridade e rápida recuperação de registros?</t>
         </is>
       </c>
-      <c r="D24" s="21" t="inlineStr">
+      <c r="D24" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E24" s="23" t="n"/>
-      <c r="F24" s="23" t="n"/>
-      <c r="G24" s="23" t="n"/>
-      <c r="H24" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Nova Solicitação de Evidência: MAQ.002.R10 - Manual de Qualidade:
-4.2.4 Controle de documentos:
-Procedimento específico, que, prevê que os documentos do QMS são adequadamente controlados quanto: Metodologia para alterações atuais, responsabilidades e métodos para aprovação, metodologia dedistribuição de versões em locais de uso, métodos para validação dosdocumentos e dados, marcação adequada em casos de retenção, bem como cuidados para manutenção no que tange a legibilidade e identificação.Preferencialmente,os  documentos  são  criados  de  forma  que  qualquer  unidade  da EssilorLuxottica possa utiliza-los, desde que possua o mesmo maquinário / equipamento envolvido. Nos casos  muito  específicos  devido  sistemas  operacionais  distintos  ou controle  e alinhamento  diferenciado com  clientes,  é  possível  criar  um  procedimento  padronizado  para  cada  unidade,  desde  que  o  mesmo respeite a hierarquia de documentos e seja controlado.
-• [Conforme] Evidencias de registros fisicos: Evidenciadas listas de presença com os treinamentos realizados.</t>
-        </is>
-      </c>
-      <c r="I24" s="19" t="n"/>
+      <c r="E24" s="154" t="n"/>
+      <c r="F24" s="154" t="n"/>
+      <c r="G24" s="154" t="n"/>
+      <c r="H24" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.017.R3 - Controle de Documentos e Registros</t>
+        </is>
+      </c>
+      <c r="I24" s="142" t="n"/>
       <c r="J24" s="128" t="n"/>
       <c r="K24" s="22" t="n"/>
       <c r="L24" s="22" t="n"/>
@@ -2424,7 +2417,7 @@
     </row>
     <row r="25" ht="23.25" customHeight="1" s="104">
       <c r="A25" s="24" t="n"/>
-      <c r="B25" s="146" t="inlineStr">
+      <c r="B25" s="136" t="inlineStr">
         <is>
           <t>RESPONSABILIDADE DA DIREÇÃO</t>
         </is>
@@ -2450,7 +2443,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="96" customHeight="1" s="104">
+    <row r="26" ht="64" customHeight="1" s="104">
       <c r="A26" s="24" t="n"/>
       <c r="B26" s="17" t="inlineStr">
         <is>
@@ -2462,42 +2455,23 @@
           <t>A alta direção fornece evidência de seu comprometimento com os requisitos do SGQ: política da qualidade, objetivos da qualidade e conduz análises críticas?</t>
         </is>
       </c>
-      <c r="D26" s="26" t="inlineStr">
+      <c r="D26" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E26" s="27" t="n"/>
-      <c r="F26" s="27" t="n"/>
-      <c r="G26" s="27" t="n"/>
-      <c r="H26" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Objetivos da Qualidade: MAQ.002.R10 - Manual da Qualidade:
-5.4 Planejamento: 
-5.4.1 Objetivos da qualidade: 
-Os objetivos da qualidade, definidos e consistentes com a política da qualidade da EssilorLuxottica, incluem o compromisso com a melhoria contínua e são medidos através de indicadores. Os  objetivos  da  qualidade  definidos  pela  Alta  Direção  são conforme (Tab.04),  sendo  monitorados mensalmente, porém com controles internos diários.
-• [Conforme] Quais são os indicadores acompanhados?: Perdas em produção - Meta &lt;= 3,5% 
-Retorno geral de clientes- Meta &lt;= 1,5%
-Service Rate(Nível de entrega no prazo) - Meta &gt;=95% - 
-Serviços em atraso com mais de 2 dias (Late Orders) - Meta &lt;=2,00% 
-Pesquisa de Satisfação - Meta &gt;= 70.00%
-• [Conforme] KPI - QUEBRA: Quebra - Meta &lt;= 3,5% - Perdas em produção
-Resultado; Conforme
-Realizado: (Maio - %) (Junho -  %) ( Julho - %)
-• [Conforme] KPI - RETORNO: Retorno - Meta &lt;= 1,5% - Retorno geral de clientes
-Resultado; Conforme
-Realizado: (Maio - %) (Junho -  %) ( Julho - %)
-• [Conforme] KPI - PESQUISA DE SATISFAÇÃO: Meta &gt;= 70.00% - Avaliação dos itens da pesquisa de satisfação do cliente.
-Realizado: 
-1. Sales Rep value of visits - 91,00%;
-2. Customer Service answers to requests  - 88,00%;
-3. Reliability of delivery dates - 76,00%;
-4. Lens Quality - 89,00%
-5. Coating Quality - 80,00%
-6. Edging e mounting - quality of the fitting</t>
-        </is>
-      </c>
-      <c r="I26" s="19" t="n"/>
+      <c r="E26" s="154" t="n"/>
+      <c r="F26" s="154" t="n"/>
+      <c r="G26" s="154" t="n"/>
+      <c r="H26" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] MAQ.002.R10 - Manual da Qualidade:
+- Política da Qualidade
+- Objetivos da Qualidade
+- Avaliação de Riscos</t>
+        </is>
+      </c>
+      <c r="I26" s="142" t="n"/>
       <c r="J26" s="128" t="n"/>
       <c r="K26" s="20">
         <f>(K25)/(K25+L25+M25)</f>
@@ -2512,7 +2486,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="96" customHeight="1" s="104">
+    <row r="27" ht="32" customHeight="1" s="104">
       <c r="A27" s="24" t="n"/>
       <c r="B27" s="17" t="inlineStr">
         <is>
@@ -2524,28 +2498,27 @@
           <t>A alta direção assegura que os requisitos regulatórios e aplicáveis sejam determinados e atendidos?</t>
         </is>
       </c>
-      <c r="D27" s="28" t="inlineStr">
+      <c r="D27" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E27" s="27" t="n"/>
-      <c r="F27" s="27" t="n"/>
-      <c r="G27" s="27" t="n"/>
-      <c r="H27" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: MAQ.002: Manual da Qualidade;
-4.SISTEMA DE GESTÃO DA QUALIDADE
-• [Conforme] Nova Solicitação de Evidência: PSQ.025.R1: Revisão Gerencial</t>
-        </is>
-      </c>
-      <c r="I27" s="19" t="n"/>
+      <c r="E27" s="154" t="n"/>
+      <c r="F27" s="154" t="n"/>
+      <c r="G27" s="154" t="n"/>
+      <c r="H27" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] MAQ.002.R10 - Manual da Qualidade:
+- Foco no Cliente</t>
+        </is>
+      </c>
+      <c r="I27" s="142" t="n"/>
       <c r="J27" s="128" t="n"/>
       <c r="K27" s="22" t="n"/>
       <c r="L27" s="22" t="n"/>
       <c r="M27" s="22" t="n"/>
     </row>
-    <row r="28" ht="96" customHeight="1" s="104">
+    <row r="28" ht="32" customHeight="1" s="104">
       <c r="A28" s="24" t="n"/>
       <c r="B28" s="17" t="inlineStr">
         <is>
@@ -2557,26 +2530,27 @@
           <t>A alta direção assegura que a política da qualidade seja aplicável, seja comunicada e compreendida e a analisa criticamente para sua contínua adequação?</t>
         </is>
       </c>
-      <c r="D28" s="28" t="inlineStr">
+      <c r="D28" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E28" s="27" t="n"/>
-      <c r="F28" s="27" t="n"/>
-      <c r="G28" s="27" t="n"/>
-      <c r="H28" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] De que forma a analise critica é realizada?: PSQ.025.R1: Revisão Gerencial</t>
-        </is>
-      </c>
-      <c r="I28" s="19" t="n"/>
+      <c r="E28" s="154" t="n"/>
+      <c r="F28" s="154" t="n"/>
+      <c r="G28" s="154" t="n"/>
+      <c r="H28" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] MAQ.002.R10 - Manual da Qualidade:
+- Política da Qualidade</t>
+        </is>
+      </c>
+      <c r="I28" s="142" t="n"/>
       <c r="J28" s="128" t="n"/>
       <c r="K28" s="22" t="n"/>
       <c r="L28" s="22" t="n"/>
       <c r="M28" s="22" t="n"/>
     </row>
-    <row r="29" ht="96" customHeight="1" s="104">
+    <row r="29" ht="32" customHeight="1" s="104">
       <c r="A29" s="24" t="n"/>
       <c r="B29" s="29" t="inlineStr">
         <is>
@@ -2588,27 +2562,27 @@
           <t>A alta direção assegura que os objetivos da qualidade, sejam estabelecidos em funções e níveis relevantes dentro da organização? Os objetivos da qualidade são mensuráveis e coerentes com a política da qualidade?</t>
         </is>
       </c>
-      <c r="D29" s="28" t="inlineStr">
+      <c r="D29" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E29" s="27" t="n"/>
-      <c r="F29" s="27" t="n"/>
-      <c r="G29" s="27" t="n"/>
-      <c r="H29" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: MAQ.002.R10: Manual da Qualidade
-• [Conforme] Nova Solicitação de Evidência: PSQ.025.R1: Revisão Gerencial</t>
-        </is>
-      </c>
-      <c r="I29" s="19" t="n"/>
+      <c r="E29" s="154" t="n"/>
+      <c r="F29" s="154" t="n"/>
+      <c r="G29" s="154" t="n"/>
+      <c r="H29" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] MAQ.002.R10 - Manual da Qualidade:
+- Objetivos da Qualidade</t>
+        </is>
+      </c>
+      <c r="I29" s="142" t="n"/>
       <c r="J29" s="128" t="n"/>
       <c r="K29" s="22" t="n"/>
       <c r="L29" s="22" t="n"/>
       <c r="M29" s="22" t="n"/>
     </row>
-    <row r="30" ht="96" customHeight="1" s="104">
+    <row r="30" ht="48" customHeight="1" s="104">
       <c r="A30" s="24" t="n"/>
       <c r="B30" s="29" t="inlineStr">
         <is>
@@ -2620,29 +2594,28 @@
           <t>A alta direção assegura que o planejamento do sistema de gestão da qualidade seja realizado de forma a satisfazer os requisitos fornecidos em 4.1, assim como os objetivos da qualidade? A integridade do sistema de gestão da qualidade é mantida quando alterações no sistema de gestão da qualidade forem planejadas e implementadas?</t>
         </is>
       </c>
-      <c r="D30" s="28" t="inlineStr">
+      <c r="D30" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E30" s="27" t="n"/>
-      <c r="F30" s="27" t="n"/>
-      <c r="G30" s="27" t="n"/>
-      <c r="H30" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Documentos Registrados: MAQ.002.R10: Manual da Qualidade:
-4. SISTEMA DE GESTÃO DA QUALIDADE:
-• [Conforme] Documentos Registrados: PSQ.028.R5 - Gestão de Riscos
-• [Conforme] Documentos Registrados: PSQ.025.R1: Revisão Gerencial</t>
-        </is>
-      </c>
-      <c r="I30" s="19" t="n"/>
+      <c r="E30" s="154" t="n"/>
+      <c r="F30" s="154" t="n"/>
+      <c r="G30" s="154" t="n"/>
+      <c r="H30" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] MAQ.002.R10 - Manual da Qualidade:
+- Planejamento do SGQ
+- Gestão de Mudança</t>
+        </is>
+      </c>
+      <c r="I30" s="142" t="n"/>
       <c r="J30" s="128" t="n"/>
       <c r="K30" s="22" t="n"/>
       <c r="L30" s="22" t="n"/>
       <c r="M30" s="22" t="n"/>
     </row>
-    <row r="31" ht="96" customHeight="1" s="104">
+    <row r="31" ht="32" customHeight="1" s="104">
       <c r="A31" s="24" t="n"/>
       <c r="B31" s="17" t="inlineStr">
         <is>
@@ -2654,26 +2627,27 @@
           <t>A alta direção documenta e assegura a inter-relação do pessoal que gerencia, desempenha e verifica o trabalho?</t>
         </is>
       </c>
-      <c r="D31" s="28" t="inlineStr">
+      <c r="D31" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E31" s="27" t="n"/>
-      <c r="F31" s="27" t="n"/>
-      <c r="G31" s="27" t="n"/>
-      <c r="H31" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: MAQ.002.R10: Manual da Qualidade:</t>
-        </is>
-      </c>
-      <c r="I31" s="19" t="n"/>
+      <c r="E31" s="154" t="n"/>
+      <c r="F31" s="154" t="n"/>
+      <c r="G31" s="154" t="n"/>
+      <c r="H31" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] MAQ.002.R10 - Manual da Qualidade:
+- Organograma e Responsabilidades</t>
+        </is>
+      </c>
+      <c r="I31" s="142" t="n"/>
       <c r="J31" s="128" t="n"/>
       <c r="K31" s="22" t="n"/>
       <c r="L31" s="22" t="n"/>
       <c r="M31" s="22" t="n"/>
     </row>
-    <row r="32" ht="25.2" customHeight="1" s="104">
+    <row r="32" ht="20" customHeight="1" s="104">
       <c r="A32" s="24" t="n"/>
       <c r="B32" s="17" t="inlineStr">
         <is>
@@ -2685,26 +2659,26 @@
           <t>A organização possui um representante da direção indicado pela alta direção?</t>
         </is>
       </c>
-      <c r="D32" s="28" t="inlineStr">
+      <c r="D32" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E32" s="27" t="n"/>
-      <c r="F32" s="27" t="n"/>
-      <c r="G32" s="27" t="n"/>
-      <c r="H32" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Nomeação do RD: FOR.118: Nomeação RD - Lealdo dos Santos</t>
-        </is>
-      </c>
-      <c r="I32" s="19" t="n"/>
+      <c r="E32" s="154" t="n"/>
+      <c r="F32" s="154" t="n"/>
+      <c r="G32" s="154" t="n"/>
+      <c r="H32" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] Nomeação do RD: FOR.118: Nomeação RD</t>
+        </is>
+      </c>
+      <c r="I32" s="142" t="n"/>
       <c r="J32" s="128" t="n"/>
       <c r="K32" s="22" t="n"/>
       <c r="L32" s="22" t="n"/>
       <c r="M32" s="22" t="n"/>
     </row>
-    <row r="33" ht="25.2" customHeight="1" s="104">
+    <row r="33" ht="20" customHeight="1" s="104">
       <c r="A33" s="24" t="n"/>
       <c r="B33" s="17" t="inlineStr">
         <is>
@@ -2716,18 +2690,26 @@
           <t>A alta direção assegura um processo de comunicação apropriado à organização com relação ao SGQ?</t>
         </is>
       </c>
-      <c r="D33" s="28" t="n"/>
-      <c r="E33" s="27" t="n"/>
-      <c r="F33" s="27" t="n"/>
-      <c r="G33" s="27" t="n"/>
-      <c r="H33" s="19" t="n"/>
-      <c r="I33" s="19" t="n"/>
+      <c r="D33" s="154" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E33" s="154" t="n"/>
+      <c r="F33" s="154" t="n"/>
+      <c r="G33" s="154" t="n"/>
+      <c r="H33" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] MAQ.002.R10 - Manual da Qualidade: Comunicação Interna</t>
+        </is>
+      </c>
+      <c r="I33" s="142" t="n"/>
       <c r="J33" s="128" t="n"/>
       <c r="K33" s="22" t="n"/>
       <c r="L33" s="22" t="n"/>
       <c r="M33" s="22" t="n"/>
     </row>
-    <row r="34" ht="25.2" customHeight="1" s="104">
+    <row r="34" ht="20" customHeight="1" s="104">
       <c r="A34" s="24" t="n"/>
       <c r="B34" s="17" t="inlineStr">
         <is>
@@ -2739,28 +2721,26 @@
           <t>A organização documentou procedimento para análise crítica pela direção?</t>
         </is>
       </c>
-      <c r="D34" s="28" t="inlineStr">
+      <c r="D34" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E34" s="27" t="n"/>
-      <c r="F34" s="27" t="n"/>
-      <c r="G34" s="27" t="n"/>
-      <c r="H34" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: MAQ.002.R10: Manual da Qualidade
-• [Conforme] Nova Solicitação de Evidência: PSQ.028.R5: Gestão de Riscos
-• [Conforme] Nova Solicitação de Evidência: PSQ.025.R1: Revisão Gerencial</t>
-        </is>
-      </c>
-      <c r="I34" s="19" t="n"/>
+      <c r="E34" s="154" t="n"/>
+      <c r="F34" s="154" t="n"/>
+      <c r="G34" s="154" t="n"/>
+      <c r="H34" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.025.R1: Revisão Gerencial: FOR.069: Ata de Reunião de Análise Crítica pela Direção</t>
+        </is>
+      </c>
+      <c r="I34" s="142" t="n"/>
       <c r="J34" s="128" t="n"/>
       <c r="K34" s="22" t="n"/>
       <c r="L34" s="22" t="n"/>
       <c r="M34" s="22" t="n"/>
     </row>
-    <row r="35" ht="96" customHeight="1" s="104">
+    <row r="35" ht="20" customHeight="1" s="104">
       <c r="A35" s="24" t="n"/>
       <c r="B35" s="17" t="inlineStr">
         <is>
@@ -2772,28 +2752,26 @@
           <t>As entradas são criticamente analisadas pela direção? (Feedback, tratamento de reclamações, comunicação às autoridades regulatórias, auditorias, monitoramento e medição de processos, monitoramento e medição de produtos, ação corretiva, ação preventiva, ações provenientes de análises anteriores, alterações que impactem o SGQ, recomendações de melhorias e requisitos regulatórios aplicáveis)</t>
         </is>
       </c>
-      <c r="D35" s="28" t="inlineStr">
+      <c r="D35" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E35" s="27" t="n"/>
-      <c r="F35" s="27" t="n"/>
-      <c r="G35" s="27" t="n"/>
-      <c r="H35" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: MAQ.002.R10: Manual da Qualidade
-• [Conforme] Nova Solicitação de Evidência: PSQ.028.R5: Gestão de Riscos
-• [Conforme] Nova Solicitação de Evidência: PSQ.025.R1: Revisão Gerencial</t>
-        </is>
-      </c>
-      <c r="I35" s="35" t="n"/>
+      <c r="E35" s="154" t="n"/>
+      <c r="F35" s="154" t="n"/>
+      <c r="G35" s="154" t="n"/>
+      <c r="H35" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.025.R1: Revisão Gerencial: FOR.069: Ata de Reunião de Análise Crítica pela Direção</t>
+        </is>
+      </c>
+      <c r="I35" s="155" t="n"/>
       <c r="J35" s="128" t="n"/>
       <c r="K35" s="22" t="n"/>
       <c r="L35" s="22" t="n"/>
       <c r="M35" s="22" t="n"/>
     </row>
-    <row r="36" ht="96" customHeight="1" s="104">
+    <row r="36" ht="20" customHeight="1" s="104">
       <c r="A36" s="24" t="n"/>
       <c r="B36" s="17" t="inlineStr">
         <is>
@@ -2805,22 +2783,20 @@
           <t>As saídas de análise crítica são registradas? (Melhorias necessárias para adequação e eficácia do SGQ, melhorias de produto, alterações para atender requisitos regulatórios, recursos)</t>
         </is>
       </c>
-      <c r="D36" s="28" t="inlineStr">
+      <c r="D36" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E36" s="27" t="n"/>
-      <c r="F36" s="27" t="n"/>
-      <c r="G36" s="27" t="n"/>
-      <c r="H36" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: MAQ.002.R10: Manual da Qualidade
-• [Conforme] Nova Solicitação de Evidência: PSQ.028.R5: Gestão de Riscos
-• [Conforme] Nova Solicitação de Evidência: PSQ.025.R1: Revisão Gerencial</t>
-        </is>
-      </c>
-      <c r="I36" s="35" t="n"/>
+      <c r="E36" s="154" t="n"/>
+      <c r="F36" s="154" t="n"/>
+      <c r="G36" s="154" t="n"/>
+      <c r="H36" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.025.R1: Revisão Gerencial: FOR.069: Ata de Reunião de Análise Crítica pela Direção</t>
+        </is>
+      </c>
+      <c r="I36" s="155" t="n"/>
       <c r="J36" s="128" t="n"/>
       <c r="K36" s="22" t="n"/>
       <c r="L36" s="22" t="n"/>
@@ -2828,7 +2804,7 @@
     </row>
     <row r="37" ht="23.25" customHeight="1" s="104">
       <c r="A37" s="24" t="n"/>
-      <c r="B37" s="146" t="inlineStr">
+      <c r="B37" s="136" t="inlineStr">
         <is>
           <t>GESTÃO DE RECURSOS</t>
         </is>
@@ -2854,7 +2830,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="96" customHeight="1" s="104">
+    <row r="38" ht="20" customHeight="1" s="104">
       <c r="A38" s="24" t="n"/>
       <c r="B38" s="17" t="inlineStr">
         <is>
@@ -2866,12 +2842,20 @@
           <t>A organização determina e provê os recursos para implementação e atendimento à requisitos regulatórios e de clientes do SGQ?</t>
         </is>
       </c>
-      <c r="D38" s="26" t="n"/>
-      <c r="E38" s="27" t="n"/>
-      <c r="F38" s="27" t="n"/>
-      <c r="G38" s="27" t="n"/>
-      <c r="H38" s="19" t="n"/>
-      <c r="I38" s="19" t="n"/>
+      <c r="D38" s="154" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E38" s="154" t="n"/>
+      <c r="F38" s="154" t="n"/>
+      <c r="G38" s="154" t="n"/>
+      <c r="H38" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] MAQ.002.R10 - Manual da Qualidade: Recursos e Infraestrutura</t>
+        </is>
+      </c>
+      <c r="I38" s="142" t="n"/>
       <c r="J38" s="128" t="n"/>
       <c r="K38" s="20">
         <f>(K37)/(K37+L37+M37)</f>
@@ -2886,7 +2870,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="50.4" customHeight="1" s="104">
+    <row r="39" ht="20" customHeight="1" s="104">
       <c r="A39" s="24" t="n"/>
       <c r="B39" s="17" t="inlineStr">
         <is>
@@ -2898,102 +2882,57 @@
           <t>O pessoal que executa o trabalho que afeta a qualidade possui competência e é treinado para a atividade que exerce? Os registros são mantidos?  A eficácia é avaliada?</t>
         </is>
       </c>
-      <c r="D39" s="28" t="inlineStr">
+      <c r="D39" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E39" s="27" t="n"/>
-      <c r="F39" s="27" t="n"/>
-      <c r="G39" s="27" t="n"/>
-      <c r="H39" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidencias de treinamento dos POPS de liberação de lentes e blocos para o colaborador Douglas Diogenes da Silva: Apresentada a lista de presença de treinamento realizado em 25/04/2025
-POP.1015.R1: Manual Operacional -Liberação de Lentes Prontas e Blocos do Estoque -Visolab (Aprovado: 15/08/2024)
-• [Conforme] Treinamento de POP de envio para LabRio - Carlos Eduardo Santos Silva: Lista de presença de treinamento realizado em 01/07/2026:
-POP.1243.R0: Manual Operacional- Serviços Direcionados para o LabRio - Visolab (Aprovado: 29/06/2026)
-• [Conforme] Treinamento de colaboradora Gabriela de jesus Santos: Lista de presença apresentada com o treinamentos realizados em 20/02/2025:
-POP.1002.R2: Manual Operacional - Rastreabilidade de pedidos - Visolab (Aprovado: 17/04/2024)
-POP.1016.R0: Manual Operacional - Aprovação e Cancelamento de Pedidos - Visolab (Aprovado: 09/02/2024)
-POP.1025.R0: Manual Operacional - Consultoria - Visolab (Aprovado: 01/04/2024)
-POP.1012.R1: Monitoramento de Realimentação do Cliente - Visolab (Aprovado: 19/08/2024)
-POP.1057.R0: Manual Operacional - Comunicação com o Cliente - Visolab (Aprovado: 18/04/2024)
-• [Conforme] [6.2] Recursos humanos: Evidências esperadas: MAQ.002 - Manual da Qualidade, 
-PSQ.023.R3: Treinamentos, 
-FOR.126 - Análise de Modos de Falhas e Efeitos (FMEA); 
-DOC.069 - Descrição de Atividade - Utilização
-• [Observação com Correção] Listas de treinamentos: As listas de presença de treinamentos da area de segurança precisam estar vinculados como padrão aos DOC.EHS presentes no qualiex.
-• [Conforme] DOC.EHS implementados pela Matriz para os laboratórios: DOC.EHS.018, DOC.EHS.020, DOC.EHS.040, DOC.EHS.042, DOC.EHS.032, DOC.EHS.039, DOC.EHS.043, DOC.EHS.045 e DOC.EHS.044
-• [Conforme] Descrição de atividades:: DOC.025.R1: DA - Operador de Produção:
-Colaborador Matheus Pereira
-Requisitos: Ensino Médio Completo ( Atendido)
-• [Não Conforme] Treinamento critico - Requer Auto-avaliação e Avaliação de Eficácia.: Observou-se que o diretório do RH não possui avaliações de eficácia:
-Registros identificados:
-Colaborador: Jhonnata Menezes da Silva Rodrigues
-Procedimento: PSQ.001
-Data: 06/04/2026
-Auto Avaliação: OK
-Avaliação de Eficácia: 06/07/2026 (Não realizada)
-Colaborador: Lais Alves Santos
-Procedimento: PSQ.001
-Data: 03/06/2026
-Auto Avaliação: OK
-Avaliação de Eficácia: 03/09/2026 (No prazo)
-• [Conforme] Controle de Competencias: PSQ.023.R3: Treinamentos
-DOC.069 -Descrição de Atividade –Utilização; 
-FOR.033 -Lista de Presença; 
-FOR.092 -Controle de Treinamento; 
-FOR.109 -Matriz de Habilidade; 
-FOR.133 -Planejamento de Treinamento; 
-FOR.141 -Auto Avaliação; 
-FOR.142 -Avaliação de Eficácia do Treinamento; 
-PSQ.017 -Controle de Documentos e Registros.
-• [Observação com Correção] 6.2. Determinar as competências necessárias para o pessoal que executa trabalho que afeta qualidade do produto: Criar um mapeamento de treinamento por Colaborador por setor, determinando quais procedimentos das diversas matrizes, o colaborador deve estar treinado.
-• [Observação com Correção] FOR.109.R5: Matriz de Habilidade: Foi observado que há campos sem preenchimento, que requerem atualização.</t>
-        </is>
-      </c>
-      <c r="I39" s="19" t="inlineStr">
-        <is>
-          <t>[OBS com Correção] As listas de presença de treinamentos da area de segurança precisam estar vinculados como padrão aos DOC.EHS presentes no qualiex.
-[OBS com Correção] Criar um mapeamento de treinamento por Colaborador por setor, determinando quais procedimentos das diversas matrizes, o colaborador deve estar treinado.
-[OBS com Correção] Foi observado que há campos sem preenchimento, que requerem atualização.</t>
-        </is>
-      </c>
+      <c r="E39" s="154" t="n"/>
+      <c r="F39" s="154" t="n"/>
+      <c r="G39" s="154" t="n"/>
+      <c r="H39" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.023.R4: Treinamentos: Matriz de Treinamento, Descrição de Cargos, Avaliação de Eficácia</t>
+        </is>
+      </c>
+      <c r="I39" s="142" t="n"/>
       <c r="J39" s="128" t="n"/>
       <c r="K39" s="22" t="n"/>
       <c r="L39" s="22" t="n"/>
       <c r="M39" s="22" t="n"/>
     </row>
-    <row r="40" ht="153.75" customHeight="1" s="104">
+    <row r="40" ht="20" customHeight="1" s="104">
       <c r="A40" s="24" t="n"/>
-      <c r="B40" s="31" t="n">
-        <v>44626</v>
+      <c r="B40" s="31" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
       </c>
       <c r="C40" s="25" t="inlineStr">
         <is>
           <t>A organização documenta os requisitos para a infraestrutura necessária para alcançar a conformidade com requisitos do produto? Previne mistura de produtos?A organização documenta os requisitos para a atividade de manutenção? Incluindo intervalo de execução, quando as atividades ou falta delas afetarem os produtos.</t>
         </is>
       </c>
-      <c r="D40" s="28" t="inlineStr">
+      <c r="D40" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E40" s="27" t="n"/>
-      <c r="F40" s="27" t="n"/>
-      <c r="G40" s="27" t="n"/>
-      <c r="H40" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Documentos: PSQ.033.R2: Procedimento de Manutenção</t>
-        </is>
-      </c>
-      <c r="I40" s="19" t="n"/>
+      <c r="E40" s="154" t="n"/>
+      <c r="F40" s="154" t="n"/>
+      <c r="G40" s="154" t="n"/>
+      <c r="H40" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.033.R2: Manutenção: Plano de Manutenção Preventiva de Equipamentos</t>
+        </is>
+      </c>
+      <c r="I40" s="142" t="n"/>
       <c r="J40" s="128" t="n"/>
       <c r="K40" s="22" t="n"/>
       <c r="L40" s="22" t="n"/>
       <c r="M40" s="22" t="n"/>
     </row>
-    <row r="41" ht="96" customHeight="1" s="104">
+    <row r="41" ht="20" customHeight="1" s="104">
       <c r="A41" s="24" t="n"/>
       <c r="B41" s="17" t="inlineStr">
         <is>
@@ -3005,29 +2944,26 @@
           <t>A organização documenta os requisitos do ambiente necessário para alcançar a conformidade com os produtos incluindo requisitos de saúde, limpeza e vestuário do pessoal que afete a qualidade do produto? O pessoal requisitado temporariamente possui competência para tal e/ou é supervisionado para tal?</t>
         </is>
       </c>
-      <c r="D41" s="28" t="inlineStr">
+      <c r="D41" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E41" s="27" t="n"/>
-      <c r="F41" s="27" t="n"/>
-      <c r="G41" s="27" t="n"/>
-      <c r="H41" s="32" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: MAQ.002 - Manual da Qualidade
-• [Conforme] MAQ.002.R10: Manual da Qualidade: 6.4 Ambiente de trabalho e controle de contaminação:
-NaEssilorLuxotticaestá disponível uma infraestrutura necessária de forma a garantir a qualidade do produto,   em   todo   o   seu   processamento,   tais   como   iluminação,   temperatura,   umidade,limpeza, armazenamento, transporte,  identificaçõese  condições  adequadas  de  atendimento  personalizado  ao cliente.
-• [Conforme] PSQ.018.R2: Realização de Produto: 6.CONTROLE AMBIENTAL</t>
-        </is>
-      </c>
-      <c r="I41" s="19" t="n"/>
+      <c r="E41" s="154" t="n"/>
+      <c r="F41" s="154" t="n"/>
+      <c r="G41" s="154" t="n"/>
+      <c r="H41" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] POP.1005.R1: Manual Operacional - Limpeza e Higienização do Laboratório</t>
+        </is>
+      </c>
+      <c r="I41" s="142" t="n"/>
       <c r="J41" s="128" t="n"/>
       <c r="K41" s="22" t="n"/>
       <c r="L41" s="22" t="n"/>
       <c r="M41" s="22" t="n"/>
     </row>
-    <row r="42" ht="96" customHeight="1" s="104">
+    <row r="42" ht="20" customHeight="1" s="104">
       <c r="A42" s="24" t="n"/>
       <c r="B42" s="17" t="inlineStr">
         <is>
@@ -3039,43 +2975,20 @@
           <t>A organização planeja e documenta as tratativas para controle de produtos contaminados ou potencialmente contaminados para previnir contaminação do ambiente de trabalho, pessoal e produtos?</t>
         </is>
       </c>
-      <c r="D42" s="28" t="inlineStr">
+      <c r="D42" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E42" s="27" t="n"/>
-      <c r="F42" s="27" t="n"/>
-      <c r="G42" s="27" t="n"/>
-      <c r="H42" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Alvará de localização e funcionamento: Secretaria Municipal
-Situação: Aberto 
-Data de início: 20/08/2007
-• [Conforme] Controle de Pragas: Empresa Q-limpo Aracaju Ambiental:
-Vigilância Sanitária - Licença de Funcionamento - N° 90/2026-SES - Validade: 04/02/2027
-Adema - Licença Simplificada - N° 9/2024 - Validade: 26/01/2027
-Serviço de Dedetização/Desratização:
-Realizado em 04/07/2026
-Validade: 04/10/2026
-• [Conforme] PGR - Programa de Gerenciamento de Riscos: REVISÃO: 
-Emitido em 30/04/2024 
-Revisão 01: 30/03/2026 
-MOTIVO: Revisão do inventário de riscos 
-Validade até: 30/03/2028
-• [Conforme] PCMSO - Programa de Controle Médico de Saúde Ocupacional: Emitido em 30/03/2026
-Validade: 30/03/2028
-• [Conforme] AVCB: CORPO DE BOMBEIROS MILITAR DE SERGIPE DIRETORIA DE ATIVIDADES TÉCNICAS
-DOCUMENTO Nº: 13364
-VALIDADE: 12/08/2026 (Vencido)
-Tratativa em andamento com os bombeiros - Protocolo 261771
-• [Conforme] LICENÇA AMBIENTAL SIMPLIFICADA: Nº: 443/2023-1 
-Data: 10/11/2023 
-Validade: 10/11/2026
-*ESTA LICENÇA É VALIDA PELO PERÍODO DE 03 (TRÊS) ANOS, CONFORME PREVISTO NO ART. 20, INCISO III DA LEI MUNICIPAL 4.594/14, E PROTOCOLO SEMA Nº 47.622/2023 DE 01 DE JUNHO DE 2023 ALTERADA PELO PARECER TÉCNICO 953/2023 DE 06 DE OUTUBRO DE 2023.</t>
-        </is>
-      </c>
-      <c r="I42" s="35" t="n"/>
+      <c r="E42" s="154" t="n"/>
+      <c r="F42" s="154" t="n"/>
+      <c r="G42" s="154" t="n"/>
+      <c r="H42" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] POP.1005.R1: Manual Operacional - Limpeza e Higienização do Laboratório</t>
+        </is>
+      </c>
+      <c r="I42" s="155" t="n"/>
       <c r="J42" s="128" t="n"/>
       <c r="K42" s="22" t="n"/>
       <c r="L42" s="22" t="n"/>
@@ -3083,7 +2996,7 @@
     </row>
     <row r="43" ht="23.25" customHeight="1" s="104">
       <c r="A43" s="24" t="n"/>
-      <c r="B43" s="146" t="inlineStr">
+      <c r="B43" s="136" t="inlineStr">
         <is>
           <t>REALIZAÇÃO DE PRODUTO (FABRICAÇÃO)</t>
         </is>
@@ -3109,7 +3022,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="106.5" customHeight="1" s="104">
+    <row r="44" ht="20" customHeight="1" s="104">
       <c r="A44" s="24" t="n"/>
       <c r="B44" s="17" t="inlineStr">
         <is>
@@ -3121,21 +3034,20 @@
           <t>A organização planeja e desenvolve processos necessários para a realização do produto? A organização documenta processos para o gerenciamento de risco?  O planejamento da realização do produto inclui os objetivos da qualidade, necessidade de estabelecer processos e documentos, atividades requeridas de verificação, validação, monitoramento, inspeção e ensaio, manuseio, armazenamento, distrubuição e rastreabilidade específicas para o produto? Os registros são armazenados?</t>
         </is>
       </c>
-      <c r="D44" s="26" t="inlineStr">
+      <c r="D44" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E44" s="27" t="n"/>
-      <c r="F44" s="27" t="n"/>
-      <c r="G44" s="27" t="n"/>
-      <c r="H44" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Procedimentos Operacionais: DOC.087.R2: Fluxograma de Processos - Visolab
-Contendo os procedimentos operacionais utilizados</t>
-        </is>
-      </c>
-      <c r="I44" s="35" t="n"/>
+      <c r="E44" s="154" t="n"/>
+      <c r="F44" s="154" t="n"/>
+      <c r="G44" s="154" t="n"/>
+      <c r="H44" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.018.R2: Realização de Produto: Fluxograma e Planejamento de Processos</t>
+        </is>
+      </c>
+      <c r="I44" s="155" t="n"/>
       <c r="J44" s="128" t="n"/>
       <c r="K44" s="20">
         <f>(K43)/(K43+L43+M43)</f>
@@ -3150,7 +3062,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="96" customHeight="1" s="104">
+    <row r="45" ht="20" customHeight="1" s="104">
       <c r="A45" s="24" t="n"/>
       <c r="B45" s="17" t="inlineStr">
         <is>
@@ -3162,30 +3074,26 @@
           <t>Os requisitos especificados pelos clientes, os não declarados, os requisitos regulatórios, treinamentos necessários para o desempenho do produto e quaisquer outro requisitos estabelecidos pela organização são determinados pela organização?</t>
         </is>
       </c>
-      <c r="D45" s="28" t="inlineStr">
+      <c r="D45" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E45" s="27" t="n"/>
-      <c r="F45" s="27" t="n"/>
-      <c r="G45" s="27" t="n"/>
-      <c r="H45" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Documentos com tratativas para esclarecimento de Requisitos.: PSQ.030.R1: Procedimento Feedback de Clientes; 
-PSQ.018.R2: Realização de Produto;
-POP.1012.R1: Monitoramento de Realimentação do Cliente - Visolab; 
-POP.1057.R0: Manual Operacional - Comunicação com o Cliente - Visolab;
-DOC.087.R2: Fluxograma de Processos - Visolab</t>
-        </is>
-      </c>
-      <c r="I45" s="35" t="n"/>
+      <c r="E45" s="154" t="n"/>
+      <c r="F45" s="154" t="n"/>
+      <c r="G45" s="154" t="n"/>
+      <c r="H45" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] POP.1057.R0: Manual Operacional - Comunicação com o Cliente - Visolab</t>
+        </is>
+      </c>
+      <c r="I45" s="155" t="n"/>
       <c r="J45" s="128" t="n"/>
       <c r="K45" s="22" t="n"/>
       <c r="L45" s="22" t="n"/>
       <c r="M45" s="22" t="n"/>
     </row>
-    <row r="46" ht="96" customHeight="1" s="104">
+    <row r="46" ht="20" customHeight="1" s="104">
       <c r="A46" s="24" t="n"/>
       <c r="B46" s="17" t="inlineStr">
         <is>
@@ -3197,31 +3105,26 @@
           <t xml:space="preserve">A organização analisa criticamente os requisitos relacionados aos produtos antes de fornecê-lo? </t>
         </is>
       </c>
-      <c r="D46" s="28" t="inlineStr">
+      <c r="D46" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E46" s="27" t="n"/>
-      <c r="F46" s="27" t="n"/>
-      <c r="G46" s="27" t="n"/>
-      <c r="H46" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Avaliação de Análise Crítica: PSQ.030.R1: Procedimento Feedback de Clientes; 
-PSQ.018.R2: Realização de Produto; 
-PSQ.001.R14: Apostila Padrão Cosmético; 
-POP.1012.R1: Monitoramento de Realimentação do Cliente - Visolab; 
-POP.1057.R0: Manual Operacional - Comunicação com o Cliente - Visolab; 
-DOC.087.R2: Fluxograma de Processos - Visolab;</t>
-        </is>
-      </c>
-      <c r="I46" s="35" t="n"/>
+      <c r="E46" s="154" t="n"/>
+      <c r="F46" s="154" t="n"/>
+      <c r="G46" s="154" t="n"/>
+      <c r="H46" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] POP.1057.R0: Manual Operacional - Comunicação com o Cliente - Visolab</t>
+        </is>
+      </c>
+      <c r="I46" s="155" t="n"/>
       <c r="J46" s="128" t="n"/>
       <c r="K46" s="22" t="n"/>
       <c r="L46" s="22" t="n"/>
       <c r="M46" s="22" t="n"/>
     </row>
-    <row r="47" ht="63" customHeight="1" s="104">
+    <row r="47" ht="20" customHeight="1" s="104">
       <c r="A47" s="24" t="n"/>
       <c r="B47" s="17" t="inlineStr">
         <is>
@@ -3233,31 +3136,26 @@
           <t>A organização planeja e documenta os arranjos de comunicação com o cliente em relação a informações do produto, tratamento de solicitações, contratos ou pedidos, feedbacks dos clientes, notas de aviso? Os registros são armazenados?</t>
         </is>
       </c>
-      <c r="D47" s="28" t="inlineStr">
+      <c r="D47" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E47" s="27" t="n"/>
-      <c r="F47" s="27" t="n"/>
-      <c r="G47" s="27" t="n"/>
-      <c r="H47" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] informações do produto e contato com o cliente: PSQ.030.R1: Procedimento Feedback de Clientes; 
-PSQ.018.R2: Realização de Produto; 
-PSQ.001.R14: Apostila Padrão Cosmético; 
-POP.1012.R1: Monitoramento de Realimentação do Cliente - Visolab; 
-POP.1057.R0: Manual Operacional - Comunicação com o Cliente - Visolab; 
-DOC.087.R2: Fluxograma de Processos - Visolab;</t>
-        </is>
-      </c>
-      <c r="I47" s="35" t="n"/>
+      <c r="E47" s="154" t="n"/>
+      <c r="F47" s="154" t="n"/>
+      <c r="G47" s="154" t="n"/>
+      <c r="H47" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] POP.1057.R0: Manual Operacional - Comunicação com o Cliente - Visolab</t>
+        </is>
+      </c>
+      <c r="I47" s="155" t="n"/>
       <c r="J47" s="128" t="n"/>
       <c r="K47" s="22" t="n"/>
       <c r="L47" s="22" t="n"/>
       <c r="M47" s="22" t="n"/>
     </row>
-    <row r="48" ht="96" customHeight="1" s="104">
+    <row r="48" ht="20" customHeight="1" s="104">
       <c r="A48" s="24" t="n"/>
       <c r="B48" s="33" t="inlineStr">
         <is>
@@ -3269,22 +3167,26 @@
           <t>A organização documenta procedimentos para projeto e desenvolvimento?</t>
         </is>
       </c>
-      <c r="D48" s="28" t="n"/>
-      <c r="E48" s="27" t="n"/>
-      <c r="F48" s="27" t="inlineStr">
+      <c r="D48" s="154" t="n"/>
+      <c r="E48" s="154" t="n"/>
+      <c r="F48" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="G48" s="27" t="n"/>
-      <c r="H48" s="34" t="n"/>
-      <c r="I48" s="35" t="n"/>
+      <c r="G48" s="154" t="n"/>
+      <c r="H48" s="144" t="inlineStr">
+        <is>
+          <t>• [Não Aplicável] Item não aplicável ao escopo de montagem e distribuição de lentes</t>
+        </is>
+      </c>
+      <c r="I48" s="155" t="n"/>
       <c r="J48" s="128" t="n"/>
       <c r="K48" s="22" t="n"/>
       <c r="L48" s="22" t="n"/>
       <c r="M48" s="22" t="n"/>
     </row>
-    <row r="49" ht="96" customHeight="1" s="104">
+    <row r="49" ht="20" customHeight="1" s="104">
       <c r="A49" s="24" t="n"/>
       <c r="B49" s="33" t="inlineStr">
         <is>
@@ -3296,22 +3198,26 @@
           <t>A organização planeja e documenta estágios de desenvolvimento, análise crítica de cada estágio do projeto, atividades de verificação, validação e transferência, as responsabilidades e autoridades, métodos de rastreabilidade e recursos necessários incluindo competências necessárias? Os registros são armazenados?</t>
         </is>
       </c>
-      <c r="D49" s="28" t="n"/>
-      <c r="E49" s="27" t="n"/>
-      <c r="F49" s="27" t="inlineStr">
+      <c r="D49" s="154" t="n"/>
+      <c r="E49" s="154" t="n"/>
+      <c r="F49" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="G49" s="27" t="n"/>
-      <c r="H49" s="34" t="n"/>
-      <c r="I49" s="35" t="n"/>
+      <c r="G49" s="154" t="n"/>
+      <c r="H49" s="144" t="inlineStr">
+        <is>
+          <t>• [Não Aplicável] Item não aplicável ao escopo de montagem e distribuição de lentes</t>
+        </is>
+      </c>
+      <c r="I49" s="155" t="n"/>
       <c r="J49" s="128" t="n"/>
       <c r="K49" s="22" t="n"/>
       <c r="L49" s="22" t="n"/>
       <c r="M49" s="22" t="n"/>
     </row>
-    <row r="50" ht="96" customHeight="1" s="104">
+    <row r="50" ht="20" customHeight="1" s="104">
       <c r="A50" s="24" t="n"/>
       <c r="B50" s="33" t="inlineStr">
         <is>
@@ -3323,22 +3229,26 @@
           <t>As entradas do produto são determinadas quanto aos seus requisitos de funcionamento, desempenho, usabilidade e segurança, os requisitos regulatórios aplicáveis, os registros do gerenciamento de risco, informações de projetos anteriores e, outros requisitos essenciais para o projeto? Os registros são armazenados?</t>
         </is>
       </c>
-      <c r="D50" s="28" t="n"/>
-      <c r="E50" s="27" t="n"/>
-      <c r="F50" s="27" t="inlineStr">
+      <c r="D50" s="154" t="n"/>
+      <c r="E50" s="154" t="n"/>
+      <c r="F50" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="G50" s="27" t="n"/>
-      <c r="H50" s="34" t="n"/>
-      <c r="I50" s="35" t="n"/>
+      <c r="G50" s="154" t="n"/>
+      <c r="H50" s="144" t="inlineStr">
+        <is>
+          <t>• [Não Aplicável] Item não aplicável ao escopo de montagem e distribuição de lentes</t>
+        </is>
+      </c>
+      <c r="I50" s="155" t="n"/>
       <c r="J50" s="128" t="n"/>
       <c r="K50" s="22" t="n"/>
       <c r="L50" s="22" t="n"/>
       <c r="M50" s="22" t="n"/>
     </row>
-    <row r="51" ht="96" customHeight="1" s="104">
+    <row r="51" ht="20" customHeight="1" s="104">
       <c r="A51" s="24" t="n"/>
       <c r="B51" s="33" t="inlineStr">
         <is>
@@ -3350,22 +3260,26 @@
           <t>As saídas de projeto atendem aos requisitos de entrada, fornece as informações apropriadas para aquisição , contem ou fazem referências a critérios de aceitação do produto, especifica as características do produto que são essencias para seu uso seguro e adequado?</t>
         </is>
       </c>
-      <c r="D51" s="28" t="n"/>
-      <c r="E51" s="27" t="n"/>
-      <c r="F51" s="27" t="inlineStr">
+      <c r="D51" s="154" t="n"/>
+      <c r="E51" s="154" t="n"/>
+      <c r="F51" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="G51" s="27" t="n"/>
-      <c r="H51" s="34" t="n"/>
-      <c r="I51" s="35" t="n"/>
+      <c r="G51" s="154" t="n"/>
+      <c r="H51" s="144" t="inlineStr">
+        <is>
+          <t>• [Não Aplicável] Item não aplicável ao escopo de montagem e distribuição de lentes</t>
+        </is>
+      </c>
+      <c r="I51" s="155" t="n"/>
       <c r="J51" s="128" t="n"/>
       <c r="K51" s="22" t="n"/>
       <c r="L51" s="22" t="n"/>
       <c r="M51" s="22" t="n"/>
     </row>
-    <row r="52" ht="96" customHeight="1" s="104">
+    <row r="52" ht="20" customHeight="1" s="104">
       <c r="A52" s="24" t="n"/>
       <c r="B52" s="33" t="inlineStr">
         <is>
@@ -3377,22 +3291,26 @@
           <t>A organização realiza análise sistemática do projeto e desenvolvimento? Os registros são armazenados?</t>
         </is>
       </c>
-      <c r="D52" s="28" t="n"/>
-      <c r="E52" s="27" t="n"/>
-      <c r="F52" s="27" t="inlineStr">
+      <c r="D52" s="154" t="n"/>
+      <c r="E52" s="154" t="n"/>
+      <c r="F52" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="G52" s="27" t="n"/>
-      <c r="H52" s="34" t="n"/>
-      <c r="I52" s="35" t="n"/>
+      <c r="G52" s="154" t="n"/>
+      <c r="H52" s="144" t="inlineStr">
+        <is>
+          <t>• [Não Aplicável] Item não aplicável ao escopo de montagem e distribuição de lentes</t>
+        </is>
+      </c>
+      <c r="I52" s="155" t="n"/>
       <c r="J52" s="128" t="n"/>
       <c r="K52" s="22" t="n"/>
       <c r="L52" s="22" t="n"/>
       <c r="M52" s="22" t="n"/>
     </row>
-    <row r="53" ht="96" customHeight="1" s="104">
+    <row r="53" ht="20" customHeight="1" s="104">
       <c r="A53" s="24" t="n"/>
       <c r="B53" s="33" t="inlineStr">
         <is>
@@ -3404,22 +3322,26 @@
           <t>A organização documenta plano de verificação do projeto e desenvolvimento? Caso o uso requeira que o produto tenha uma interface com outro produto, a verificação deve atender os requisitos dessa interação?</t>
         </is>
       </c>
-      <c r="D53" s="28" t="n"/>
-      <c r="E53" s="27" t="n"/>
-      <c r="F53" s="27" t="inlineStr">
+      <c r="D53" s="154" t="n"/>
+      <c r="E53" s="154" t="n"/>
+      <c r="F53" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="G53" s="27" t="n"/>
-      <c r="H53" s="34" t="n"/>
-      <c r="I53" s="35" t="n"/>
+      <c r="G53" s="154" t="n"/>
+      <c r="H53" s="144" t="inlineStr">
+        <is>
+          <t>• [Não Aplicável] Item não aplicável ao escopo de montagem e distribuição de lentes</t>
+        </is>
+      </c>
+      <c r="I53" s="155" t="n"/>
       <c r="J53" s="128" t="n"/>
       <c r="K53" s="22" t="n"/>
       <c r="L53" s="22" t="n"/>
       <c r="M53" s="22" t="n"/>
     </row>
-    <row r="54" ht="96" customHeight="1" s="104">
+    <row r="54" ht="20" customHeight="1" s="104">
       <c r="A54" s="24" t="n"/>
       <c r="B54" s="33" t="inlineStr">
         <is>
@@ -3431,22 +3353,26 @@
           <t>A organização executa a validação em produto representativo (protótipo)? Atende aos requisitos do produto?</t>
         </is>
       </c>
-      <c r="D54" s="28" t="n"/>
-      <c r="E54" s="27" t="n"/>
-      <c r="F54" s="27" t="inlineStr">
+      <c r="D54" s="154" t="n"/>
+      <c r="E54" s="154" t="n"/>
+      <c r="F54" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="G54" s="27" t="n"/>
-      <c r="H54" s="34" t="n"/>
-      <c r="I54" s="35" t="n"/>
+      <c r="G54" s="154" t="n"/>
+      <c r="H54" s="144" t="inlineStr">
+        <is>
+          <t>• [Não Aplicável] Item não aplicável ao escopo de montagem e distribuição de lentes</t>
+        </is>
+      </c>
+      <c r="I54" s="155" t="n"/>
       <c r="J54" s="128" t="n"/>
       <c r="K54" s="22" t="n"/>
       <c r="L54" s="22" t="n"/>
       <c r="M54" s="22" t="n"/>
     </row>
-    <row r="55" ht="96" customHeight="1" s="104">
+    <row r="55" ht="20" customHeight="1" s="104">
       <c r="A55" s="24" t="n"/>
       <c r="B55" s="33" t="inlineStr">
         <is>
@@ -3458,22 +3384,26 @@
           <t xml:space="preserve">A organização documenta procedimento para a transferência do projeto para fabricação? </t>
         </is>
       </c>
-      <c r="D55" s="28" t="n"/>
-      <c r="E55" s="27" t="n"/>
-      <c r="F55" s="27" t="inlineStr">
+      <c r="D55" s="154" t="n"/>
+      <c r="E55" s="154" t="n"/>
+      <c r="F55" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="G55" s="27" t="n"/>
-      <c r="H55" s="34" t="n"/>
-      <c r="I55" s="35" t="n"/>
+      <c r="G55" s="154" t="n"/>
+      <c r="H55" s="144" t="inlineStr">
+        <is>
+          <t>• [Não Aplicável] Item não aplicável ao escopo de montagem e distribuição de lentes</t>
+        </is>
+      </c>
+      <c r="I55" s="155" t="n"/>
       <c r="J55" s="128" t="n"/>
       <c r="K55" s="22" t="n"/>
       <c r="L55" s="22" t="n"/>
       <c r="M55" s="22" t="n"/>
     </row>
-    <row r="56" ht="96" customHeight="1" s="104">
+    <row r="56" ht="20" customHeight="1" s="104">
       <c r="A56" s="24" t="n"/>
       <c r="B56" s="33" t="inlineStr">
         <is>
@@ -3485,22 +3415,26 @@
           <t>A organização documenta procedimento para controlar alterações de projeto e desenvolvimento? Antes da implementação elas são analisadas, verificadas, validadas e aprovadas?</t>
         </is>
       </c>
-      <c r="D56" s="28" t="n"/>
-      <c r="E56" s="27" t="n"/>
-      <c r="F56" s="27" t="inlineStr">
+      <c r="D56" s="154" t="n"/>
+      <c r="E56" s="154" t="n"/>
+      <c r="F56" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="G56" s="27" t="n"/>
-      <c r="H56" s="34" t="n"/>
-      <c r="I56" s="35" t="n"/>
+      <c r="G56" s="154" t="n"/>
+      <c r="H56" s="144" t="inlineStr">
+        <is>
+          <t>• [Não Aplicável] Item não aplicável ao escopo de montagem e distribuição de lentes</t>
+        </is>
+      </c>
+      <c r="I56" s="155" t="n"/>
       <c r="J56" s="128" t="n"/>
       <c r="K56" s="22" t="n"/>
       <c r="L56" s="22" t="n"/>
       <c r="M56" s="22" t="n"/>
     </row>
-    <row r="57" ht="96" customHeight="1" s="104">
+    <row r="57" ht="20" customHeight="1" s="104">
       <c r="A57" s="24" t="n"/>
       <c r="B57" s="33" t="inlineStr">
         <is>
@@ -3512,22 +3446,26 @@
           <t xml:space="preserve">A organização mantem arquivo do projeto e desenvolvimento para cada tipo de produto ou família? </t>
         </is>
       </c>
-      <c r="D57" s="28" t="n"/>
-      <c r="E57" s="27" t="n"/>
-      <c r="F57" s="27" t="inlineStr">
+      <c r="D57" s="154" t="n"/>
+      <c r="E57" s="154" t="n"/>
+      <c r="F57" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="G57" s="27" t="n"/>
-      <c r="H57" s="34" t="n"/>
-      <c r="I57" s="35" t="n"/>
+      <c r="G57" s="154" t="n"/>
+      <c r="H57" s="144" t="inlineStr">
+        <is>
+          <t>• [Não Aplicável] Item não aplicável ao escopo de montagem e distribuição de lentes</t>
+        </is>
+      </c>
+      <c r="I57" s="155" t="n"/>
       <c r="J57" s="128" t="n"/>
       <c r="K57" s="22" t="n"/>
       <c r="L57" s="22" t="n"/>
       <c r="M57" s="22" t="n"/>
     </row>
-    <row r="58" ht="63" customHeight="1" s="104">
+    <row r="58" ht="32" customHeight="1" s="104">
       <c r="A58" s="24" t="n"/>
       <c r="B58" s="17" t="inlineStr">
         <is>
@@ -3539,27 +3477,27 @@
           <t>A organização documenta procedimento para aquisição de produtos? O procedimento estabelece critérios de avaliação e seleção de fornecedores? A organização realiza acompanhamento do fornecedor qualificado? Os registros são armazenados?</t>
         </is>
       </c>
-      <c r="D58" s="28" t="inlineStr">
+      <c r="D58" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E58" s="27" t="n"/>
-      <c r="F58" s="27" t="n"/>
-      <c r="G58" s="27" t="n"/>
-      <c r="H58" s="35" t="inlineStr">
-        <is>
-          <t>• [Conforme] Procedimento da qualidade para gestão de fornecedores: PSQ.020.R7: Gestão de Fornecedores;
-• [Conforme] Manual de compras: DOC.085.R0 - Manual de compras;</t>
-        </is>
-      </c>
-      <c r="I58" s="35" t="n"/>
+      <c r="E58" s="154" t="n"/>
+      <c r="F58" s="154" t="n"/>
+      <c r="G58" s="154" t="n"/>
+      <c r="H58" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.018.R2: Realização de Produto: FOR.146: Lista de Fornecedores Qualificados
+• [Conforme] FOR.147: Avaliação e Reavaliação de Fornecedores</t>
+        </is>
+      </c>
+      <c r="I58" s="155" t="n"/>
       <c r="J58" s="128" t="n"/>
       <c r="K58" s="22" t="n"/>
       <c r="L58" s="22" t="n"/>
       <c r="M58" s="22" t="n"/>
     </row>
-    <row r="59" ht="96" customHeight="1" s="104">
+    <row r="59" ht="20" customHeight="1" s="104">
       <c r="A59" s="24" t="n"/>
       <c r="B59" s="17" t="inlineStr">
         <is>
@@ -3571,28 +3509,26 @@
           <t>A organização mantem informações de aquisição dos produtos que constem as especificações, requisitos de aceitação e requisitos do pessoal e SGQ? Os registros são armazenados corretamente?</t>
         </is>
       </c>
-      <c r="D59" s="28" t="inlineStr">
+      <c r="D59" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E59" s="27" t="n"/>
-      <c r="F59" s="27" t="n"/>
-      <c r="G59" s="27" t="n"/>
-      <c r="H59" s="35" t="inlineStr">
-        <is>
-          <t>• [Conforme] Avaliações de fornecedores - MultiOptica SP: FOR.127 -Avaliação e Seleção de Fornecedor;
-FOR.136 -Reavaliação de Fornecedor;
-FOR.148 -Monitoramento Anual de Desempenho de Fornecedor;</t>
-        </is>
-      </c>
-      <c r="I59" s="35" t="n"/>
+      <c r="E59" s="154" t="n"/>
+      <c r="F59" s="154" t="n"/>
+      <c r="G59" s="154" t="n"/>
+      <c r="H59" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] DOC.085.R0: Manual de Compras - Visolab</t>
+        </is>
+      </c>
+      <c r="I59" s="155" t="n"/>
       <c r="J59" s="128" t="n"/>
       <c r="K59" s="22" t="n"/>
       <c r="L59" s="22" t="n"/>
       <c r="M59" s="22" t="n"/>
     </row>
-    <row r="60" ht="96" customHeight="1" s="104">
+    <row r="60" ht="20" customHeight="1" s="104">
       <c r="A60" s="24" t="n"/>
       <c r="B60" s="17" t="inlineStr">
         <is>
@@ -3604,29 +3540,26 @@
           <t>A organização realiza verificação nos produtos adquiridos? Existe procedimento para a atividade? Caso seja realizada vistoria nas instalações do fornecedor, é informado na informação de aquisição os itens verificados e critérios de aceitação?</t>
         </is>
       </c>
-      <c r="D60" s="28" t="inlineStr">
+      <c r="D60" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E60" s="27" t="n"/>
-      <c r="F60" s="27" t="n"/>
-      <c r="G60" s="27" t="n"/>
-      <c r="H60" s="35" t="inlineStr">
-        <is>
-          <t>• [Conforme] Procedimentos: PSQ.020 - Gestão de Fornecedores; 
-FOR.126 - Análise de Modos de Falhas e Efeitos (FMEA); 
-FOR.127 - Avaliação e Seleção de Fornecedor; 
-POP.364 - Inspeção de Recebimento dos Vernizes e Primers</t>
-        </is>
-      </c>
-      <c r="I60" s="35" t="n"/>
+      <c r="E60" s="154" t="n"/>
+      <c r="F60" s="154" t="n"/>
+      <c r="G60" s="154" t="n"/>
+      <c r="H60" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] POP.1122.R0: Manual Operacional - Recebimento de Lentes e Blocos - Visolab</t>
+        </is>
+      </c>
+      <c r="I60" s="155" t="n"/>
       <c r="J60" s="128" t="n"/>
       <c r="K60" s="22" t="n"/>
       <c r="L60" s="22" t="n"/>
       <c r="M60" s="22" t="n"/>
     </row>
-    <row r="61" ht="63" customHeight="1" s="104">
+    <row r="61" ht="32" customHeight="1" s="104">
       <c r="A61" s="24" t="n"/>
       <c r="B61" s="17" t="inlineStr">
         <is>
@@ -3638,36 +3571,27 @@
           <t>Caso a organização forneça um serviço, este é planejado, monitorado e controlado para que se assegure conformidade com especificações? Existe procedimentos documentados para isso? Os registros são armazenados devidamente?</t>
         </is>
       </c>
-      <c r="D61" s="28" t="inlineStr">
+      <c r="D61" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E61" s="27" t="n"/>
-      <c r="F61" s="27" t="n"/>
-      <c r="G61" s="27" t="n"/>
-      <c r="H61" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] PSQ.033.R2: Procedimento de Manutenção: 1.OBJETIVO
-Este  procedimento  descreve  as  atividades,  responsabilidade  e  imperativos  estratégicos  necessários  para  e execução efetiva da Metodologia de Manutenção Regional (RMM)•O  objetivo  principal  do  RMM  é  obter  a  utilização  ideal  dos principais  equipamentos  do  processo  de fabricação. Isso é feito garantindo sistematicamente:
-•Condições de operação seguras
-•Qualidade e conformidade de processos
-•Confiabilidade e disponibilidade operacional
-•Redução de custos 
-Através dos principais pilares: manutenção planejada (preventiva e preditiva), gestão de fornecedores e peças de reposição, educação e treinamento, transformação e padronização e utilidades e infraestrutura.
-• [Conforme] PSQ.029.R3: Procedimento de Gestão de Mudança: 1.OBJETIVO: 
-Estabelecer a metodologia que permita adaptar de forma detalhada as mudanças que influenciam o sistema de gestão da qualidade. Desde a identificação, diagnóstico, controle, adaptação e planejamento adequado.
-2.ESCOPO: 
-Aplica-se a mudanças geradas por necessidades ou solicitações que afetam o sistema de gestão da qualidade. Da mesma forma, os riscos e oportunidades identificados em cada um dos processos.</t>
-        </is>
-      </c>
-      <c r="I61" s="35" t="n"/>
+      <c r="E61" s="154" t="n"/>
+      <c r="F61" s="154" t="n"/>
+      <c r="G61" s="154" t="n"/>
+      <c r="H61" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] POP.1002.R1: Manual Operacional - Rastreabilidade de Pedidos Visolab
+• [Conforme] Instruções de Trabalho da Linha de Produção</t>
+        </is>
+      </c>
+      <c r="I61" s="155" t="n"/>
       <c r="J61" s="128" t="n"/>
       <c r="K61" s="22" t="n"/>
       <c r="L61" s="22" t="n"/>
       <c r="M61" s="22" t="n"/>
     </row>
-    <row r="62" ht="96" customHeight="1" s="104">
+    <row r="62" ht="20" customHeight="1" s="104">
       <c r="A62" s="24" t="n"/>
       <c r="B62" s="17" t="inlineStr">
         <is>
@@ -3679,27 +3603,26 @@
           <t>A organização documenta requisitos para limpeza ou controle de contaminação do produto? Esterilização, limpeza antes do uso, limpeza pós-uso?</t>
         </is>
       </c>
-      <c r="D62" s="28" t="inlineStr">
+      <c r="D62" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E62" s="27" t="n"/>
-      <c r="F62" s="27" t="n"/>
-      <c r="G62" s="27" t="n"/>
-      <c r="H62" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Nova Solicitação de Evidência: MAQ.002.R10: Manual da Qualidade; 
-DOC.EHS.030.R0: Avaliação Química da Concentração dos Contaminantes;</t>
-        </is>
-      </c>
-      <c r="I62" s="19" t="n"/>
+      <c r="E62" s="154" t="n"/>
+      <c r="F62" s="154" t="n"/>
+      <c r="G62" s="154" t="n"/>
+      <c r="H62" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] POP.1005.R1: Manual Operacional - Limpeza e Higienização do Laboratório</t>
+        </is>
+      </c>
+      <c r="I62" s="142" t="n"/>
       <c r="J62" s="128" t="n"/>
       <c r="K62" s="22" t="n"/>
       <c r="L62" s="22" t="n"/>
       <c r="M62" s="22" t="n"/>
     </row>
-    <row r="63" ht="96" customHeight="1" s="104">
+    <row r="63" ht="20" customHeight="1" s="104">
       <c r="A63" s="24" t="n"/>
       <c r="B63" s="33" t="inlineStr">
         <is>
@@ -3711,22 +3634,26 @@
           <t>Caso haja produtos que necessitem ser instalados, a organização documentou requisitos de instalação e critérios de aceitação? Caso a instalação seja realizada por empresa terceira, há processo de qualificação da mesma?</t>
         </is>
       </c>
-      <c r="D63" s="28" t="n"/>
-      <c r="E63" s="27" t="n"/>
-      <c r="F63" s="27" t="inlineStr">
+      <c r="D63" s="154" t="n"/>
+      <c r="E63" s="154" t="n"/>
+      <c r="F63" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="G63" s="27" t="n"/>
-      <c r="H63" s="19" t="n"/>
-      <c r="I63" s="35" t="n"/>
+      <c r="G63" s="154" t="n"/>
+      <c r="H63" s="144" t="inlineStr">
+        <is>
+          <t>• [Não Aplicável] Não aplicável (produtos não estéreis)</t>
+        </is>
+      </c>
+      <c r="I63" s="155" t="n"/>
       <c r="J63" s="128" t="n"/>
       <c r="K63" s="22" t="n"/>
       <c r="L63" s="22" t="n"/>
       <c r="M63" s="22" t="n"/>
     </row>
-    <row r="64" ht="96" customHeight="1" s="104">
+    <row r="64" ht="20" customHeight="1" s="104">
       <c r="A64" s="24" t="n"/>
       <c r="B64" s="33" t="inlineStr">
         <is>
@@ -3738,18 +3665,26 @@
           <t>A organização documenta procedimento para assistência técnica de produtos? Especifica os critérios de aceitação? Os registros são devidamente mantidos?</t>
         </is>
       </c>
-      <c r="D64" s="28" t="n"/>
-      <c r="E64" s="27" t="n"/>
-      <c r="F64" s="27" t="n"/>
-      <c r="G64" s="27" t="n"/>
-      <c r="H64" s="19" t="n"/>
-      <c r="I64" s="35" t="n"/>
+      <c r="D64" s="154" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E64" s="154" t="n"/>
+      <c r="F64" s="154" t="n"/>
+      <c r="G64" s="154" t="n"/>
+      <c r="H64" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.018.R2: Realização de Produto: Parâmetros de Montagem</t>
+        </is>
+      </c>
+      <c r="I64" s="155" t="n"/>
       <c r="J64" s="128" t="n"/>
       <c r="K64" s="22" t="n"/>
       <c r="L64" s="22" t="n"/>
       <c r="M64" s="22" t="n"/>
     </row>
-    <row r="65" ht="96" customHeight="1" s="104">
+    <row r="65" ht="20" customHeight="1" s="104">
       <c r="A65" s="24" t="n"/>
       <c r="B65" s="33" t="inlineStr">
         <is>
@@ -3761,22 +3696,26 @@
           <t>A organização mantem os registros dos parâmetros para processos de esterilização para cada lote de produto? Os registros são devidamente armazenados?</t>
         </is>
       </c>
-      <c r="D65" s="28" t="n"/>
-      <c r="E65" s="27" t="n"/>
-      <c r="F65" s="27" t="inlineStr">
+      <c r="D65" s="154" t="n"/>
+      <c r="E65" s="154" t="n"/>
+      <c r="F65" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="G65" s="27" t="n"/>
-      <c r="H65" s="19" t="n"/>
-      <c r="I65" s="35" t="n"/>
+      <c r="G65" s="154" t="n"/>
+      <c r="H65" s="144" t="inlineStr">
+        <is>
+          <t>• [Não Aplicável] Não aplicável (não há produtos estéreis)</t>
+        </is>
+      </c>
+      <c r="I65" s="155" t="n"/>
       <c r="J65" s="128" t="n"/>
       <c r="K65" s="22" t="n"/>
       <c r="L65" s="22" t="n"/>
       <c r="M65" s="22" t="n"/>
     </row>
-    <row r="66" ht="96" customHeight="1" s="104">
+    <row r="66" ht="20" customHeight="1" s="104">
       <c r="A66" s="24" t="n"/>
       <c r="B66" s="17" t="inlineStr">
         <is>
@@ -3788,27 +3727,26 @@
           <t xml:space="preserve">A organização possui procedimento para validação de qualquer processo de produção e fornecimento como software e outras ferramentas que sejam necessárias? O procedimento possui critérios de avaliação, qualificação de equipamentos e pessoal, técnicas estatísticas, requisitos de registros, etc.? </t>
         </is>
       </c>
-      <c r="D66" s="28" t="inlineStr">
+      <c r="D66" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E66" s="27" t="n"/>
-      <c r="F66" s="27" t="n"/>
-      <c r="G66" s="27" t="n"/>
-      <c r="H66" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] PSQ.027.R2: Procedimento de Validação: 2.4 Validação de Software:
-A  validação  dos  softwares,devem  demonstrar  a  habilidade  destes  processos  em  alcançar  os resultados  planejados  de  maneira  consistenteincluindo, critérios  definidos  para  análise  crítica  e aprovação  dos  processos, qualificação  de  equipamentos  e  pessoal, uso  de  métodos,  procedimentos  e critérios  de  aceitação  específicos,  controle  de  amostras  quando  aplicáveis,  requisitos  para  registros  e aprovações  para  alterações  de  processos.Estes  estudos  e  validações  devem  ser  controlados e registrados.</t>
-        </is>
-      </c>
-      <c r="I66" s="35" t="n"/>
+      <c r="E66" s="154" t="n"/>
+      <c r="F66" s="154" t="n"/>
+      <c r="G66" s="154" t="n"/>
+      <c r="H66" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.027.R2: Validação: Validação de Processos Produtivos</t>
+        </is>
+      </c>
+      <c r="I66" s="155" t="n"/>
       <c r="J66" s="128" t="n"/>
       <c r="K66" s="22" t="n"/>
       <c r="L66" s="22" t="n"/>
       <c r="M66" s="22" t="n"/>
     </row>
-    <row r="67" ht="96" customHeight="1" s="104">
+    <row r="67" ht="20" customHeight="1" s="104">
       <c r="A67" s="24" t="n"/>
       <c r="B67" s="33" t="inlineStr">
         <is>
@@ -3820,22 +3758,26 @@
           <t xml:space="preserve">A organização documenta procedimento para validação de processo de esterilização e barreira estéril? </t>
         </is>
       </c>
-      <c r="D67" s="28" t="n"/>
-      <c r="E67" s="27" t="n"/>
-      <c r="F67" s="27" t="inlineStr">
+      <c r="D67" s="154" t="n"/>
+      <c r="E67" s="154" t="n"/>
+      <c r="F67" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="G67" s="27" t="n"/>
-      <c r="H67" s="19" t="n"/>
-      <c r="I67" s="35" t="n"/>
+      <c r="G67" s="154" t="n"/>
+      <c r="H67" s="144" t="inlineStr">
+        <is>
+          <t>• [Não Aplicável] Não aplicável (não há esterilização)</t>
+        </is>
+      </c>
+      <c r="I67" s="155" t="n"/>
       <c r="J67" s="128" t="n"/>
       <c r="K67" s="22" t="n"/>
       <c r="L67" s="22" t="n"/>
       <c r="M67" s="22" t="n"/>
     </row>
-    <row r="68" ht="96" customHeight="1" s="104">
+    <row r="68" ht="20" customHeight="1" s="104">
       <c r="A68" s="24" t="n"/>
       <c r="B68" s="17" t="inlineStr">
         <is>
@@ -3847,29 +3789,26 @@
           <t>A organização documenta procedimento para identificação dos produtos em todas as etapas de produção e distribuição? Os produtos em situação de quarentena e não conforme são identificados impossibilitando seu uso intensional?</t>
         </is>
       </c>
-      <c r="D68" s="28" t="inlineStr">
+      <c r="D68" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E68" s="27" t="n"/>
-      <c r="F68" s="27" t="n"/>
-      <c r="G68" s="27" t="n"/>
-      <c r="H68" s="36" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: MAQ.002.R10 - Manual da Qualidade; 
-PSQ.026.R1 - Identificação e Rastreabilidade; 
-PSQ.018.R2 - Realização de Produto; 
-DOC.087.R2 - fluxograma de Processos</t>
-        </is>
-      </c>
-      <c r="I68" s="35" t="n"/>
+      <c r="E68" s="154" t="n"/>
+      <c r="F68" s="154" t="n"/>
+      <c r="G68" s="154" t="n"/>
+      <c r="H68" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.026.R1: Identificação e Rastreabilidade</t>
+        </is>
+      </c>
+      <c r="I68" s="155" t="n"/>
       <c r="J68" s="128" t="n"/>
       <c r="K68" s="22" t="n"/>
       <c r="L68" s="22" t="n"/>
       <c r="M68" s="22" t="n"/>
     </row>
-    <row r="69" ht="96" customHeight="1" s="104">
+    <row r="69" ht="20" customHeight="1" s="104">
       <c r="A69" s="24" t="n"/>
       <c r="B69" s="17" t="inlineStr">
         <is>
@@ -3881,28 +3820,26 @@
           <t>A organização documenta procedimento de rastreabilidade dos produtos?</t>
         </is>
       </c>
-      <c r="D69" s="28" t="inlineStr">
+      <c r="D69" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E69" s="27" t="n"/>
-      <c r="F69" s="27" t="n"/>
-      <c r="G69" s="27" t="n"/>
-      <c r="H69" s="36" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: MAQ.002.R10 - Manual da Qualidade; 
-PSQ.018.R2 - Realização de Produto; Fluxograma de Processos
-POP.1002.R1 - Manual Operacional - Rastreabilidade de Pedidos Visolab</t>
-        </is>
-      </c>
-      <c r="I69" s="35" t="n"/>
+      <c r="E69" s="154" t="n"/>
+      <c r="F69" s="154" t="n"/>
+      <c r="G69" s="154" t="n"/>
+      <c r="H69" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.026.R1: Identificação e Rastreabilidade: Rastreabilidade por Ordem de Serviço</t>
+        </is>
+      </c>
+      <c r="I69" s="155" t="n"/>
       <c r="J69" s="128" t="n"/>
       <c r="K69" s="22" t="n"/>
       <c r="L69" s="22" t="n"/>
       <c r="M69" s="22" t="n"/>
     </row>
-    <row r="70" ht="96" customHeight="1" s="104">
+    <row r="70" ht="20" customHeight="1" s="104">
       <c r="A70" s="24" t="n"/>
       <c r="B70" s="33" t="inlineStr">
         <is>
@@ -3914,22 +3851,26 @@
           <t>A organização mantem registros dos produtos de saúde implantáveis? Há exigência para que os distribuidores mantenham registros de rastreabilidade dos produtos?</t>
         </is>
       </c>
-      <c r="D70" s="28" t="n"/>
-      <c r="E70" s="27" t="n"/>
-      <c r="F70" s="27" t="inlineStr">
+      <c r="D70" s="154" t="n"/>
+      <c r="E70" s="154" t="n"/>
+      <c r="F70" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="G70" s="27" t="n"/>
-      <c r="H70" s="19" t="n"/>
-      <c r="I70" s="35" t="n"/>
+      <c r="G70" s="154" t="n"/>
+      <c r="H70" s="144" t="inlineStr">
+        <is>
+          <t>• [Não Aplicável] Não aplicável (dispositivos médicos não implantáveis)</t>
+        </is>
+      </c>
+      <c r="I70" s="155" t="n"/>
       <c r="J70" s="128" t="n"/>
       <c r="K70" s="22" t="n"/>
       <c r="L70" s="22" t="n"/>
       <c r="M70" s="22" t="n"/>
     </row>
-    <row r="71" ht="96" customHeight="1" s="104">
+    <row r="71" ht="20" customHeight="1" s="104">
       <c r="A71" s="24" t="n"/>
       <c r="B71" s="17" t="inlineStr">
         <is>
@@ -3941,31 +3882,26 @@
           <t>A organização identifica, verifica, protege e resguarda itens de propriedade do cliente como contratos, documentos e registros?Isso é comunicado ao cliente?</t>
         </is>
       </c>
-      <c r="D71" s="28" t="inlineStr">
+      <c r="D71" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E71" s="27" t="n"/>
-      <c r="F71" s="27" t="n"/>
-      <c r="G71" s="27" t="n"/>
-      <c r="H71" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] PSQ.019.R2: Preservação de Insumo e Produto: 1.OBJETIVO: 
-Determinar  os  procedimentos  para  identificar,  verificar,  proteger,  garantira  preservação  de  conformidade  do insumo  e  produto durante  o  processamento,  armazenamento,  manuseio  e  distribuição. Dessa forma,  proteger o insumo e produto contra qualquer tipo de alteração, contaminação e/ou danos.
-2.ESCOPO: 
-Aplica-se  para as  atividades  de produção,  armazenamento e distribuição de lentes  oftálmicas  EssilorLuxottica, cobrindo o ciclo de vida do produto.
-• [Conforme] POP.1003.R1: Manual Operacional - Casamento de Armação - Visolab: 2. RECEBIMENTO DE ARMAÇÕES
-Pedido 951514_0 acompanhamento com estojo disponibilizado pelo laboratório.</t>
-        </is>
-      </c>
-      <c r="I71" s="35" t="n"/>
+      <c r="E71" s="154" t="n"/>
+      <c r="F71" s="154" t="n"/>
+      <c r="G71" s="154" t="n"/>
+      <c r="H71" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.018.R2: Realização de Produto: Controle de Propriedade do Cliente</t>
+        </is>
+      </c>
+      <c r="I71" s="155" t="n"/>
       <c r="J71" s="128" t="n"/>
       <c r="K71" s="22" t="n"/>
       <c r="L71" s="22" t="n"/>
       <c r="M71" s="22" t="n"/>
     </row>
-    <row r="72" ht="63" customHeight="1" s="104">
+    <row r="72" ht="20" customHeight="1" s="104">
       <c r="A72" s="24" t="n"/>
       <c r="B72" s="17" t="inlineStr">
         <is>
@@ -3977,27 +3913,26 @@
           <t>A organização documenta procedimento para preservação do produto durante as etapas de processamento, armazenamento, manuseio e distribuição? Alem das condições de acondicionamento, há proteção na identificação dos produtos?</t>
         </is>
       </c>
-      <c r="D72" s="28" t="inlineStr">
+      <c r="D72" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E72" s="27" t="n"/>
-      <c r="F72" s="27" t="n"/>
-      <c r="G72" s="27" t="n"/>
-      <c r="H72" s="19" t="inlineStr">
-        <is>
-          <t>• [Conforme] Procedimentos: PSQ.019 - Preservação de Insumo e Produto; 
-Manual Operacional - Casamento de Armação</t>
-        </is>
-      </c>
-      <c r="I72" s="35" t="n"/>
+      <c r="E72" s="154" t="n"/>
+      <c r="F72" s="154" t="n"/>
+      <c r="G72" s="154" t="n"/>
+      <c r="H72" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.019.R2: Preservação de Insumo e Produto</t>
+        </is>
+      </c>
+      <c r="I72" s="155" t="n"/>
       <c r="J72" s="128" t="n"/>
       <c r="K72" s="22" t="n"/>
       <c r="L72" s="22" t="n"/>
       <c r="M72" s="22" t="n"/>
     </row>
-    <row r="73" ht="96" customHeight="1" s="104">
+    <row r="73" ht="20" customHeight="1" s="104">
       <c r="A73" s="24" t="n"/>
       <c r="B73" s="17" t="inlineStr">
         <is>
@@ -4009,38 +3944,20 @@
           <t>A organização determina o monitoramento e a medição nos equipamentos de monitoramento e medição dos produtos? Há uma verificação sistemática e periódica? Os registros são devidamente armazenados? Os equipamentos são identificados? Os equipamentos são protegidos contra danos, deterioração durante manuseio, manutenção e armazenamento?</t>
         </is>
       </c>
-      <c r="D73" s="28" t="inlineStr">
+      <c r="D73" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E73" s="27" t="n"/>
-      <c r="F73" s="27" t="n"/>
-      <c r="G73" s="27" t="n"/>
-      <c r="H73" s="37" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: PSQ.032.R7: Monitoramento de Equipamento de Medição, 
-FOR.151.R1: Análise Crítica do Certificado de Calibração, 
-POP.891.R0: Manual Operacional - Análise Crítica dos Certificados de Calibração, FOR.152.R1: Etiqueta de Calibração
-• [Conforme] Procedimento da Qualidade: PSQ.032.R7: Monitoramento de Equipamento de Medição
-• [Conforme] Evidencia de Calibração (VI-01): Instrumento Viscosímetro 
-Tag: VI-01
-Certificado: 33846/2026
-Calibrado em: 16/04/2026
-Vencimento em: 16/04/2027
-• [Conforme] Evidencia de Calibração (DE-01): Instrumento: Densimetro
-Tag: DE-01
-Certificado: 33839/2026
-Calibrado em: 17/04/2026
-Vencimento em: 17/04/2027
-• [Conforme] Evidencia de Calibração (LE-02): Instrumento Lensometro 
-Tag: LE-02
-Certificado: VIS-0002/2026
-Calibrado em: 08/04/2026
-Vencimento em: 08/10/2026</t>
-        </is>
-      </c>
-      <c r="I73" s="35" t="n"/>
+      <c r="E73" s="154" t="n"/>
+      <c r="F73" s="154" t="n"/>
+      <c r="G73" s="154" t="n"/>
+      <c r="H73" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.032.R7: Monitoramento de Equipamento de Medição: Calibração de Lensômetros e Paquímetros</t>
+        </is>
+      </c>
+      <c r="I73" s="155" t="n"/>
       <c r="J73" s="128" t="n"/>
       <c r="K73" s="22" t="n"/>
       <c r="L73" s="22" t="n"/>
@@ -4048,7 +3965,7 @@
     </row>
     <row r="74" ht="23.25" customHeight="1" s="104">
       <c r="A74" s="24" t="n"/>
-      <c r="B74" s="146" t="inlineStr">
+      <c r="B74" s="136" t="inlineStr">
         <is>
           <t>MEDIÇÃO, ANÁLISE E MELHORIA</t>
         </is>
@@ -4074,7 +3991,7 @@
         <v/>
       </c>
     </row>
-    <row r="75" ht="96" customHeight="1" s="104">
+    <row r="75" ht="20" customHeight="1" s="104">
       <c r="A75" s="24" t="n"/>
       <c r="B75" s="17" t="inlineStr">
         <is>
@@ -4086,32 +4003,20 @@
           <t>A organização planeja e implementa processos de monitoramento, medição, análise e melhoria que demonstrem e assegurem a eficácia dos produtos e SGQ?</t>
         </is>
       </c>
-      <c r="D75" s="26" t="inlineStr">
+      <c r="D75" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E75" s="27" t="n"/>
-      <c r="F75" s="27" t="n"/>
-      <c r="G75" s="27" t="n"/>
-      <c r="H75" s="35" t="inlineStr">
-        <is>
-          <t>• [Conforme] MAQ.002.R10: Manual da Qualidade: 8.MEDIÇÃO, ANÁLISE E MELHORIA
-• [Conforme] PSQ.030.R1: Procedimento Feedback de Clientes: 6.3 Tratamento de reclamações:
-Um relatório, FOR.071 -Formulário RNC -Relatório de Não Conformidade, é gerado quando se obtêm na Pesquisa de Satisfação do Cliente do Grupo Essilor os três piores índices de satisfação abaixo de 70%. É realizado também um plano de ação com o objetivo de melhoria do nível de satisfação. Projetos de melhoria também podem ser realizados com o objetivo principal de atender os requisitos do cliente.
-• [Conforme] PSQ.018.R2: Realização de Produto: 5.DESCRIÇÃO DAS ATIVIDADES
-• [Conforme] PSQ.022.R5: Não Conformidade - Ações Corretivas e Preventivas: 5. DISPOSIÇÕES: 
-5.1 Monitoramento e medição de processo 
-5.2 Monitoramento e medição de produto 
-5.3 Controle de produto não conforme 
-5.4 Ações em resposta ao produto não conforme detectado antes da entrega
-5.5 Ações em resposta ao produto não conforme detectado após a entrega
-5.6 Retrabalhos
-5.7 Identificação de potenciais problemas
-5.8 Análise de dados -Tratativas de não conformidades e melhorias</t>
-        </is>
-      </c>
-      <c r="I75" s="35" t="n"/>
+      <c r="E75" s="154" t="n"/>
+      <c r="F75" s="154" t="n"/>
+      <c r="G75" s="154" t="n"/>
+      <c r="H75" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.018.R2: Realização de Produto: Plano de Inspeção e Controle de Qualidade</t>
+        </is>
+      </c>
+      <c r="I75" s="155" t="n"/>
       <c r="J75" s="128" t="n"/>
       <c r="K75" s="20">
         <f>(K74)/(K74+L74+M74)</f>
@@ -4126,7 +4031,7 @@
         <v/>
       </c>
     </row>
-    <row r="76" ht="96" customHeight="1" s="104">
+    <row r="76" ht="32" customHeight="1" s="104">
       <c r="A76" s="24" t="n"/>
       <c r="B76" s="17" t="inlineStr">
         <is>
@@ -4138,31 +4043,27 @@
           <t xml:space="preserve">A organização documenta procedimento para realimentação (feedback, sugestões, reclamações, dúvidas)? Determina e monitora informações de atendimento as especificações dos clientes? </t>
         </is>
       </c>
-      <c r="D76" s="28" t="inlineStr">
+      <c r="D76" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E76" s="27" t="n"/>
-      <c r="F76" s="27" t="n"/>
-      <c r="G76" s="27" t="n"/>
-      <c r="H76" s="91" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: PSQ.030.R1: Procedimento Feedback de Clientes; 
-PSQ.018.R2: Realização de Produto; 
-PSQ.022.R5: Não Conformidade - Ações Corretivas e Preventivas; 
-MAQ.002.R10: Manual da Qualidade; 
-POP.1012: Monitoramento de Realimentação do Cliente - Visolab;
-POP.1057.R0: Manual Operacional - Comunicação com o Cliente - Visolab;</t>
-        </is>
-      </c>
-      <c r="I76" s="35" t="n"/>
+      <c r="E76" s="154" t="n"/>
+      <c r="F76" s="154" t="n"/>
+      <c r="G76" s="154" t="n"/>
+      <c r="H76" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] POP.1012.R1: Monitoramento de Realimentação do Cliente - Visolab
+• [Conforme] Pesquisa Anual de Satisfação</t>
+        </is>
+      </c>
+      <c r="I76" s="155" t="n"/>
       <c r="J76" s="128" t="n"/>
       <c r="K76" s="22" t="n"/>
       <c r="L76" s="22" t="n"/>
       <c r="M76" s="22" t="n"/>
     </row>
-    <row r="77" ht="75.59999999999999" customHeight="1" s="104">
+    <row r="77" ht="20" customHeight="1" s="104">
       <c r="A77" s="24" t="n"/>
       <c r="B77" s="17" t="inlineStr">
         <is>
@@ -4174,31 +4075,26 @@
           <t>A organização documenta procedimento para tratamento de reclamações? O tempo de resposta atende às especificações dos clientes e requisitos regulatórios? Documenta procedimento para ações corretivas e preventivas provenientes de investigações de reclamações?</t>
         </is>
       </c>
-      <c r="D77" s="28" t="inlineStr">
+      <c r="D77" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E77" s="27" t="n"/>
-      <c r="F77" s="27" t="n"/>
-      <c r="G77" s="27" t="n"/>
-      <c r="H77" s="35" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: PSQ.030.R1: Procedimento Feedback de Clientes; 
-PSQ.018.R2: Realização de Produto; 
-PSQ.022.R5: Não Conformidade - Ações Corretivas e Preventivas; 
-MAQ.002.R10: Manual da Qualidade; 
-POP.1012: Monitoramento de Realimentação do Cliente - Visolab;
-POP.1057.R0: Manual Operacional - Comunicação com o Cliente - Visolab;</t>
-        </is>
-      </c>
-      <c r="I77" s="35" t="n"/>
+      <c r="E77" s="154" t="n"/>
+      <c r="F77" s="154" t="n"/>
+      <c r="G77" s="154" t="n"/>
+      <c r="H77" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] POP.1057.R0: Manual Operacional - Comunicação com o Cliente - Visolab</t>
+        </is>
+      </c>
+      <c r="I77" s="155" t="n"/>
       <c r="J77" s="128" t="n"/>
       <c r="K77" s="22" t="n"/>
       <c r="L77" s="22" t="n"/>
       <c r="M77" s="22" t="n"/>
     </row>
-    <row r="78" ht="96" customHeight="1" s="104">
+    <row r="78" ht="48" customHeight="1" s="104">
       <c r="A78" s="24" t="n"/>
       <c r="B78" s="17" t="inlineStr">
         <is>
@@ -4210,15 +4106,397 @@
           <t>A organização documenta procedimento para notificação às autoridades provenientes de ações relacionadas ao produto? Evento adverso, alterações importantes, recolhimento. Os registros são mantidos conforme item 4.2.5?</t>
         </is>
       </c>
-      <c r="D78" s="150" t="inlineStr">
+      <c r="D78" s="154" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E78" s="27" t="n"/>
-      <c r="F78" s="27" t="n"/>
-      <c r="G78" s="27" t="n"/>
-      <c r="H78" s="148" t="inlineStr">
+      <c r="E78" s="154" t="n"/>
+      <c r="F78" s="154" t="n"/>
+      <c r="G78" s="154" t="n"/>
+      <c r="H78" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.022.R5: Não Conformidade - Ações Corretivas e Preventivas
+• [Conforme] POP.1057.R0: Tratativa de Reclamações
+• [Conforme] POP.1012.R1: Realimentação de Clientes</t>
+        </is>
+      </c>
+      <c r="I78" s="156" t="n"/>
+      <c r="J78" s="128" t="n"/>
+      <c r="K78" s="22" t="n"/>
+      <c r="L78" s="22" t="n"/>
+      <c r="M78" s="22" t="n"/>
+    </row>
+    <row r="79" ht="20" customHeight="1" s="104">
+      <c r="A79" s="24" t="n"/>
+      <c r="B79" s="17" t="inlineStr">
+        <is>
+          <t>8.2.4</t>
+        </is>
+      </c>
+      <c r="C79" s="25" t="inlineStr">
+        <is>
+          <t>A organização possui procedimento para auditoria interna? As autoridades são definidas? Os registros são mantidos? É realizado acompanhamento de atividades apontadas em outras auditorias?</t>
+        </is>
+      </c>
+      <c r="D79" s="154" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E79" s="154" t="n"/>
+      <c r="F79" s="154" t="n"/>
+      <c r="G79" s="154" t="n"/>
+      <c r="H79" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.024.R3: Auditoria: FOR.140: Relatório de Auditoria Interna, FOR.123: Agenda, FOR.167: Cronograma, FOR.143: Check List</t>
+        </is>
+      </c>
+      <c r="I79" s="155" t="n"/>
+      <c r="J79" s="128" t="n"/>
+      <c r="K79" s="22" t="n"/>
+      <c r="L79" s="22" t="n"/>
+      <c r="M79" s="22" t="n"/>
+    </row>
+    <row r="80" ht="20" customHeight="1" s="104">
+      <c r="A80" s="24" t="n"/>
+      <c r="B80" s="17" t="inlineStr">
+        <is>
+          <t>8.2.5</t>
+        </is>
+      </c>
+      <c r="C80" s="25" t="inlineStr">
+        <is>
+          <t>É realizado monitoramento e medição dos processos do SGQ? Possui KPIs? Os resultados planejados que não forem alcançados, são realizadas correções e ações corretivas?</t>
+        </is>
+      </c>
+      <c r="D80" s="154" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E80" s="154" t="n"/>
+      <c r="F80" s="154" t="n"/>
+      <c r="G80" s="154" t="n"/>
+      <c r="H80" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] MAQ.002.R10: Manual da Qualidade - Monitoramento dos Objetivos da Qualidade</t>
+        </is>
+      </c>
+      <c r="I80" s="155" t="n"/>
+      <c r="J80" s="128" t="n"/>
+      <c r="K80" s="22" t="n"/>
+      <c r="L80" s="22" t="n"/>
+      <c r="M80" s="22" t="n"/>
+    </row>
+    <row r="81" ht="20" customHeight="1" s="104">
+      <c r="A81" s="24" t="n"/>
+      <c r="B81" s="17" t="inlineStr">
+        <is>
+          <t>8.2.6</t>
+        </is>
+      </c>
+      <c r="C81" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A organização monitora características e requisitos do produto? É realizado registro dos responsáveis por liberação do produto para fim de rastreabilidade? </t>
+        </is>
+      </c>
+      <c r="D81" s="154" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E81" s="154" t="n"/>
+      <c r="F81" s="154" t="n"/>
+      <c r="G81" s="154" t="n"/>
+      <c r="H81" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] Inspeção Final de Montagem: FOR.089: Registro de Inspeção de Produtos Acabados</t>
+        </is>
+      </c>
+      <c r="I81" s="155" t="n"/>
+      <c r="J81" s="128" t="n"/>
+      <c r="K81" s="22" t="n"/>
+      <c r="L81" s="22" t="n"/>
+      <c r="M81" s="22" t="n"/>
+    </row>
+    <row r="82" ht="20" customHeight="1" s="104">
+      <c r="A82" s="24" t="n"/>
+      <c r="B82" s="17" t="inlineStr">
+        <is>
+          <t>8.3.1</t>
+        </is>
+      </c>
+      <c r="C82" s="25" t="inlineStr">
+        <is>
+          <t>A organização documenta procedimento para identificação, responsabilidades e tratativas de produtos não conforme? Assegura que produtos não conforme sejam controlados prevenindo seu uso ou entrega não intensional? Os registros são mantidos?</t>
+        </is>
+      </c>
+      <c r="D82" s="154" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E82" s="154" t="n"/>
+      <c r="F82" s="154" t="n"/>
+      <c r="G82" s="154" t="n"/>
+      <c r="H82" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.022.R5: Não Conformidade - Ações Corretivas e Preventivas</t>
+        </is>
+      </c>
+      <c r="I82" s="155" t="n"/>
+      <c r="J82" s="128" t="n"/>
+      <c r="K82" s="22" t="n"/>
+      <c r="L82" s="22" t="n"/>
+      <c r="M82" s="22" t="n"/>
+    </row>
+    <row r="83" ht="20" customHeight="1" s="104">
+      <c r="A83" s="24" t="n"/>
+      <c r="B83" s="17" t="inlineStr">
+        <is>
+          <t>8.3.2</t>
+        </is>
+      </c>
+      <c r="C83" s="25" t="inlineStr">
+        <is>
+          <t>Para produto não conforme detectado antes da entrega, a organização assegura método para sanar a não conformidade liberando o produto para uso ou segregando-o quando seu uso não for possível?</t>
+        </is>
+      </c>
+      <c r="D83" s="154" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E83" s="154" t="n"/>
+      <c r="F83" s="154" t="n"/>
+      <c r="G83" s="154" t="n"/>
+      <c r="H83" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.022.R5: Não Conformidade - Segregação e Identificação de Produtos NC</t>
+        </is>
+      </c>
+      <c r="I83" s="155" t="n"/>
+      <c r="J83" s="128" t="n"/>
+      <c r="K83" s="22" t="n"/>
+      <c r="L83" s="22" t="n"/>
+      <c r="M83" s="22" t="n"/>
+    </row>
+    <row r="84" ht="20" customHeight="1" s="104">
+      <c r="A84" s="24" t="n"/>
+      <c r="B84" s="17" t="inlineStr">
+        <is>
+          <t>8.3.3</t>
+        </is>
+      </c>
+      <c r="C84" s="25" t="inlineStr">
+        <is>
+          <t>A organização adota ações apropriadas aos efeitos ou efeitos potencias do produto não conforme após a entrega ou início do uso?
+Possui procedimentos para a emissão de notas de aviso? Os registros são mantidos?</t>
+        </is>
+      </c>
+      <c r="D84" s="154" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E84" s="154" t="n"/>
+      <c r="F84" s="154" t="n"/>
+      <c r="G84" s="154" t="n"/>
+      <c r="H84" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.022.R5: Não Conformidade - Disposição de Produtos NC</t>
+        </is>
+      </c>
+      <c r="I84" s="155" t="n"/>
+      <c r="J84" s="128" t="n"/>
+      <c r="K84" s="22" t="n"/>
+      <c r="L84" s="22" t="n"/>
+      <c r="M84" s="22" t="n"/>
+    </row>
+    <row r="85" ht="20" customHeight="1" s="104">
+      <c r="A85" s="24" t="n"/>
+      <c r="B85" s="17" t="inlineStr">
+        <is>
+          <t>8.3.4</t>
+        </is>
+      </c>
+      <c r="C85" s="25" t="inlineStr">
+        <is>
+          <t>A organização executa retrabalho? São realizados de acordo com procedimentos documentados? Os produtos são verificados após  o retrabalho para assegurar que ele atenda critérios de aceitação e requisitos regulatórios aplicáveis?</t>
+        </is>
+      </c>
+      <c r="D85" s="154" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E85" s="154" t="n"/>
+      <c r="F85" s="154" t="n"/>
+      <c r="G85" s="154" t="n"/>
+      <c r="H85" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.022.R5: Não Conformidade - Retrabalho e Reinspeção</t>
+        </is>
+      </c>
+      <c r="I85" s="155" t="n"/>
+      <c r="J85" s="128" t="n"/>
+      <c r="K85" s="22" t="n"/>
+      <c r="L85" s="22" t="n"/>
+      <c r="M85" s="22" t="n"/>
+    </row>
+    <row r="86" ht="20" customHeight="1" s="104">
+      <c r="A86" s="24" t="n"/>
+      <c r="B86" s="17" t="inlineStr">
+        <is>
+          <t>8.4</t>
+        </is>
+      </c>
+      <c r="C86" s="25" t="inlineStr">
+        <is>
+          <t>A organização documenta procedimento para determinar coleta e análise de dados referente a reclamações, feedbacks, requisitos regulatórios, fornecedores, auditorias, relatórios de serviços e tratá-los?</t>
+        </is>
+      </c>
+      <c r="D86" s="154" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E86" s="154" t="n"/>
+      <c r="F86" s="154" t="n"/>
+      <c r="G86" s="154" t="n"/>
+      <c r="H86" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.025.R1: Revisão Gerencial - Análise de Dados e Indicadores de Processos</t>
+        </is>
+      </c>
+      <c r="I86" s="155" t="n"/>
+      <c r="J86" s="128" t="n"/>
+      <c r="K86" s="22" t="n"/>
+      <c r="L86" s="22" t="n"/>
+      <c r="M86" s="22" t="n"/>
+    </row>
+    <row r="87" ht="32" customHeight="1" s="104">
+      <c r="A87" s="24" t="n"/>
+      <c r="B87" s="17" t="inlineStr">
+        <is>
+          <t>8.5.1</t>
+        </is>
+      </c>
+      <c r="C87" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A organização identifica e implementa ações para assegurar melhoria contínua do SGQ e outros processos relacionados ao produto? </t>
+        </is>
+      </c>
+      <c r="D87" s="154" t="n"/>
+      <c r="E87" s="154" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F87" s="154" t="n"/>
+      <c r="G87" s="154" t="n"/>
+      <c r="H87" s="144" t="inlineStr">
+        <is>
+          <t>• [Não Conforme] KPI - SERVICE RATE: Meta &gt;=95% | Realizado: Junho: 91,17%
+• [Não Conforme] KPI - LATE ORDERS: Meta &lt;=2,00% | Realizado: Junho: 4,32%</t>
+        </is>
+      </c>
+      <c r="I87" s="144" t="inlineStr">
+        <is>
+          <t>Abertura de Plano de Ação para desvios de metas em Junho.</t>
+        </is>
+      </c>
+      <c r="J87" s="128" t="n"/>
+      <c r="K87" s="22" t="n"/>
+      <c r="L87" s="22" t="n"/>
+      <c r="M87" s="22" t="n"/>
+    </row>
+    <row r="88" ht="20" customHeight="1" s="104">
+      <c r="A88" s="24" t="n"/>
+      <c r="B88" s="17" t="inlineStr">
+        <is>
+          <t>8.5.2</t>
+        </is>
+      </c>
+      <c r="C88" s="25" t="inlineStr">
+        <is>
+          <t>A organização possui procedimento para ações corretivas que aborde a análise das não conformidades, avalia a necessidade de ações para que elas não recorram, necessidade de atualização de documentação e analise eficácia da ação adotada?</t>
+        </is>
+      </c>
+      <c r="D88" s="154" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E88" s="154" t="n"/>
+      <c r="F88" s="154" t="n"/>
+      <c r="G88" s="154" t="n"/>
+      <c r="H88" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.022.R5: Não Conformidade - Ações Corretivas: FOR.062: Registro de Não Conformidade (RNC)</t>
+        </is>
+      </c>
+      <c r="I88" s="155" t="n"/>
+      <c r="J88" s="128" t="n"/>
+      <c r="K88" s="22" t="n"/>
+      <c r="L88" s="22" t="n"/>
+      <c r="M88" s="22" t="n"/>
+    </row>
+    <row r="89" ht="20" customHeight="1" s="104">
+      <c r="A89" s="24" t="n"/>
+      <c r="B89" s="17" t="inlineStr">
+        <is>
+          <t>8.5.3</t>
+        </is>
+      </c>
+      <c r="C89" s="25" t="inlineStr">
+        <is>
+          <t>A organização determina ações para eliminar causas de não conformidades potênciais? Possui procedimento para para determinação de não conformidades potenciais, avalia a necessidade de ações para prevenir novas não conformidades, planeja e documenta ações necessárias e as implementa conforme apropriado?</t>
+        </is>
+      </c>
+      <c r="D89" s="154" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E89" s="154" t="n"/>
+      <c r="F89" s="154" t="n"/>
+      <c r="G89" s="154" t="n"/>
+      <c r="H89" s="144" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.022.R5: Não Conformidade - Ações Preventivas e Gestão de Riscos (PSQ.028)</t>
+        </is>
+      </c>
+      <c r="I89" s="155" t="n"/>
+      <c r="J89" s="128" t="n"/>
+      <c r="K89" s="22" t="n"/>
+      <c r="L89" s="22" t="n"/>
+      <c r="M89" s="22" t="n"/>
+    </row>
+    <row r="90" ht="15.75" customHeight="1" s="104">
+      <c r="A90" s="5" t="n"/>
+      <c r="B90" s="7" t="n"/>
+      <c r="C90" s="38" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D90" s="140">
+        <f>COUNTIF(D14:D89,"X")</f>
+        <v/>
+      </c>
+      <c r="E90" s="141">
+        <f>D90/($D$93)</f>
+        <v/>
+      </c>
+      <c r="F90" s="142" t="inlineStr">
+        <is>
+          <t>Itens Conformes</t>
+        </is>
+      </c>
+      <c r="G90" s="143" t="n"/>
+      <c r="H90" s="144" t="inlineStr">
         <is>
           <t>• [Conforme] PSQ.022.R5: Não Conformidade - Ações Corretivas e Preventivas: A organização deve realizar o acompanhamento de todas as soluções de problemas e oportunidades de melhorias criadas para que o sistema de qualidade esteja em constante melhoria dos seus processos. Neste sentido, é obrigatório inserir todos os registros relacionados no Controle Anual de Registros: Plano de Ação, RNC, 8D, Gestão de Mudança e Revisão Gerencial.
 • [Conforme] POP.1057.R0: Manual Operacional - Comunicação com o Cliente - Visolab: 2. RECLAMAÇÕES: 
@@ -4232,33 +4510,34 @@
 4. PESQUISA ANUAL DE SATISFAÇÃO</t>
         </is>
       </c>
-      <c r="I78" s="136" t="n"/>
-      <c r="J78" s="128" t="n"/>
-      <c r="K78" s="22" t="n"/>
-      <c r="L78" s="22" t="n"/>
-      <c r="M78" s="22" t="n"/>
-    </row>
-    <row r="79" ht="123" customHeight="1" s="104">
-      <c r="A79" s="24" t="n"/>
-      <c r="B79" s="17" t="inlineStr">
-        <is>
-          <t>8.2.4</t>
-        </is>
-      </c>
-      <c r="C79" s="25" t="inlineStr">
-        <is>
-          <t>A organização possui procedimento para auditoria interna? As autoridades são definidas? Os registros são mantidos? É realizado acompanhamento de atividades apontadas em outras auditorias?</t>
-        </is>
-      </c>
-      <c r="D79" s="150" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E79" s="27" t="n"/>
-      <c r="F79" s="27" t="n"/>
-      <c r="G79" s="27" t="n"/>
-      <c r="H79" s="148" t="inlineStr">
+      <c r="I90" s="145" t="n"/>
+      <c r="K90" s="5" t="n"/>
+      <c r="L90" s="5" t="n"/>
+      <c r="M90" s="5" t="n"/>
+    </row>
+    <row r="91" ht="15.75" customHeight="1" s="104">
+      <c r="A91" s="5" t="n"/>
+      <c r="B91" s="7" t="n"/>
+      <c r="C91" s="38" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="D91" s="140">
+        <f>COUNTIF(E14:E89,"X")</f>
+        <v/>
+      </c>
+      <c r="E91" s="141">
+        <f>D91/($D$93)</f>
+        <v/>
+      </c>
+      <c r="F91" s="142" t="inlineStr">
+        <is>
+          <t>Itens Não Conformes</t>
+        </is>
+      </c>
+      <c r="G91" s="143" t="n"/>
+      <c r="H91" s="144" t="inlineStr">
         <is>
           <t>• [Conforme] PSQ.024.R3: Auditoria: FOR.140: Relatório de Auditoria Interna, 
 FOR.123: Agenda de Auditoria, 
@@ -4266,65 +4545,67 @@
 FOR.143: Formulário de Check List da Auditoria ISO 1348</t>
         </is>
       </c>
-      <c r="I79" s="35" t="n"/>
-      <c r="J79" s="128" t="n"/>
-      <c r="K79" s="22" t="n"/>
-      <c r="L79" s="22" t="n"/>
-      <c r="M79" s="22" t="n"/>
-    </row>
-    <row r="80" ht="96" customHeight="1" s="104">
-      <c r="A80" s="24" t="n"/>
-      <c r="B80" s="17" t="inlineStr">
-        <is>
-          <t>8.2.5</t>
-        </is>
-      </c>
-      <c r="C80" s="25" t="inlineStr">
-        <is>
-          <t>É realizado monitoramento e medição dos processos do SGQ? Possui KPIs? Os resultados planejados que não forem alcançados, são realizadas correções e ações corretivas?</t>
-        </is>
-      </c>
-      <c r="D80" s="150" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E80" s="27" t="n"/>
-      <c r="F80" s="27" t="n"/>
-      <c r="G80" s="27" t="n"/>
-      <c r="H80" s="148" t="inlineStr">
+      <c r="I91" s="145" t="n"/>
+      <c r="K91" s="5" t="n"/>
+      <c r="L91" s="5" t="n"/>
+      <c r="M91" s="5" t="n"/>
+    </row>
+    <row r="92" ht="15.75" customHeight="1" s="104">
+      <c r="A92" s="5" t="n"/>
+      <c r="B92" s="7" t="n"/>
+      <c r="C92" s="38" t="inlineStr">
+        <is>
+          <t>OM</t>
+        </is>
+      </c>
+      <c r="D92" s="140">
+        <f>COUNTIF(G14:G89,"X")</f>
+        <v/>
+      </c>
+      <c r="E92" s="141">
+        <f>D92/($D$93)</f>
+        <v/>
+      </c>
+      <c r="F92" s="142" t="inlineStr">
+        <is>
+          <t>Oportunidade de Melhoria</t>
+        </is>
+      </c>
+      <c r="G92" s="143" t="n"/>
+      <c r="H92" s="144" t="inlineStr">
         <is>
           <t>• [Conforme] Evidências / Documentos Registrados: MAQ.002.R10 - Manual da Qualidade:
 - Objetivos da Qualidade</t>
         </is>
       </c>
-      <c r="I80" s="35" t="n"/>
-      <c r="J80" s="128" t="n"/>
-      <c r="K80" s="22" t="n"/>
-      <c r="L80" s="22" t="n"/>
-      <c r="M80" s="22" t="n"/>
-    </row>
-    <row r="81" ht="96" customHeight="1" s="104">
-      <c r="A81" s="24" t="n"/>
-      <c r="B81" s="17" t="inlineStr">
-        <is>
-          <t>8.2.6</t>
-        </is>
-      </c>
-      <c r="C81" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A organização monitora características e requisitos do produto? É realizado registro dos responsáveis por liberação do produto para fim de rastreabilidade? </t>
-        </is>
-      </c>
-      <c r="D81" s="150" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E81" s="27" t="n"/>
-      <c r="F81" s="27" t="n"/>
-      <c r="G81" s="27" t="n"/>
-      <c r="H81" s="148" t="inlineStr">
+      <c r="I92" s="145" t="n"/>
+      <c r="K92" s="5" t="n"/>
+      <c r="L92" s="5" t="n"/>
+      <c r="M92" s="5" t="n"/>
+    </row>
+    <row r="93" ht="15.75" customHeight="1" s="104">
+      <c r="A93" s="5" t="n"/>
+      <c r="B93" s="7" t="n"/>
+      <c r="C93" s="38" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="D93" s="140">
+        <f>SUM(D90:D92)</f>
+        <v/>
+      </c>
+      <c r="E93" s="141">
+        <f>SUM(E90:E92)</f>
+        <v/>
+      </c>
+      <c r="F93" s="142" t="inlineStr">
+        <is>
+          <t>TOTAL de Itens Auditados</t>
+        </is>
+      </c>
+      <c r="G93" s="143" t="n"/>
+      <c r="H93" s="144" t="inlineStr">
         <is>
           <t>• [Conforme] Evidências / Documentos Registrados: PSQ.018.R2 - Realização de Produto; 
 PSQ.017.R3 - Controle de Documentos e Registros; 
@@ -4343,459 +4624,7 @@
 POP.1002.R1 - Manual Operacional - Rastreabilidade de Pedidos Visolab</t>
         </is>
       </c>
-      <c r="I81" s="35" t="n"/>
-      <c r="J81" s="128" t="n"/>
-      <c r="K81" s="22" t="n"/>
-      <c r="L81" s="22" t="n"/>
-      <c r="M81" s="22" t="n"/>
-    </row>
-    <row r="82" ht="96" customHeight="1" s="104">
-      <c r="A82" s="24" t="n"/>
-      <c r="B82" s="17" t="inlineStr">
-        <is>
-          <t>8.3.1</t>
-        </is>
-      </c>
-      <c r="C82" s="25" t="inlineStr">
-        <is>
-          <t>A organização documenta procedimento para identificação, responsabilidades e tratativas de produtos não conforme? Assegura que produtos não conforme sejam controlados prevenindo seu uso ou entrega não intensional? Os registros são mantidos?</t>
-        </is>
-      </c>
-      <c r="D82" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E82" s="27" t="n"/>
-      <c r="F82" s="27" t="n"/>
-      <c r="G82" s="27" t="n"/>
-      <c r="H82" s="35" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: PSQ.018.R2: Realização de Produto; 
-PSQ.022.R5: Não Conformidade - Ações Corretivas e Preventivas; 
-POP.1001.R3: Manual Operacional - Produtos e Insumos Não Conforme - Visolab;</t>
-        </is>
-      </c>
-      <c r="I82" s="35" t="n"/>
-      <c r="J82" s="128" t="n"/>
-      <c r="K82" s="22" t="n"/>
-      <c r="L82" s="22" t="n"/>
-      <c r="M82" s="22" t="n"/>
-    </row>
-    <row r="83" ht="96" customHeight="1" s="104">
-      <c r="A83" s="24" t="n"/>
-      <c r="B83" s="17" t="inlineStr">
-        <is>
-          <t>8.3.2</t>
-        </is>
-      </c>
-      <c r="C83" s="25" t="inlineStr">
-        <is>
-          <t>Para produto não conforme detectado antes da entrega, a organização assegura método para sanar a não conformidade liberando o produto para uso ou segregando-o quando seu uso não for possível?</t>
-        </is>
-      </c>
-      <c r="D83" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E83" s="27" t="n"/>
-      <c r="F83" s="27" t="n"/>
-      <c r="G83" s="27" t="n"/>
-      <c r="H83" s="35" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: PSQ.018.R2: Realização de Produto; 
-PSQ.022.R5: Não Conformidade - Ações Corretivas e Preventivas; 
-POP.1001.R3: Manual Operacional - Produtos e Insumos Não Conforme - Visolab;</t>
-        </is>
-      </c>
-      <c r="I83" s="35" t="n"/>
-      <c r="J83" s="128" t="n"/>
-      <c r="K83" s="22" t="n"/>
-      <c r="L83" s="22" t="n"/>
-      <c r="M83" s="22" t="n"/>
-    </row>
-    <row r="84" ht="63" customHeight="1" s="104">
-      <c r="A84" s="24" t="n"/>
-      <c r="B84" s="17" t="inlineStr">
-        <is>
-          <t>8.3.3</t>
-        </is>
-      </c>
-      <c r="C84" s="25" t="inlineStr">
-        <is>
-          <t>A organização adota ações apropriadas aos efeitos ou efeitos potencias do produto não conforme após a entrega ou início do uso?
-Possui procedimentos para a emissão de notas de aviso? Os registros são mantidos?</t>
-        </is>
-      </c>
-      <c r="D84" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E84" s="27" t="n"/>
-      <c r="F84" s="27" t="n"/>
-      <c r="G84" s="27" t="n"/>
-      <c r="H84" s="35" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: PSQ.018.R2: Realização de Produto; 
-PSQ.022.R5: Não Conformidade - Ações Corretivas e Preventivas; 
-POP.1001.R3: Manual Operacional - Produtos e Insumos Não Conforme - Visolab;</t>
-        </is>
-      </c>
-      <c r="I84" s="35" t="n"/>
-      <c r="J84" s="128" t="n"/>
-      <c r="K84" s="22" t="n"/>
-      <c r="L84" s="22" t="n"/>
-      <c r="M84" s="22" t="n"/>
-    </row>
-    <row r="85" ht="96" customHeight="1" s="104">
-      <c r="A85" s="24" t="n"/>
-      <c r="B85" s="17" t="inlineStr">
-        <is>
-          <t>8.3.4</t>
-        </is>
-      </c>
-      <c r="C85" s="25" t="inlineStr">
-        <is>
-          <t>A organização executa retrabalho? São realizados de acordo com procedimentos documentados? Os produtos são verificados após  o retrabalho para assegurar que ele atenda critérios de aceitação e requisitos regulatórios aplicáveis?</t>
-        </is>
-      </c>
-      <c r="D85" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E85" s="27" t="n"/>
-      <c r="F85" s="27" t="n"/>
-      <c r="G85" s="27" t="n"/>
-      <c r="H85" s="35" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: PSQ.022.R5: Não Conformidade - Ações Corretivas e Preventivas;</t>
-        </is>
-      </c>
-      <c r="I85" s="35" t="n"/>
-      <c r="J85" s="128" t="n"/>
-      <c r="K85" s="22" t="n"/>
-      <c r="L85" s="22" t="n"/>
-      <c r="M85" s="22" t="n"/>
-    </row>
-    <row r="86" ht="96" customHeight="1" s="104">
-      <c r="A86" s="24" t="n"/>
-      <c r="B86" s="17" t="inlineStr">
-        <is>
-          <t>8.4</t>
-        </is>
-      </c>
-      <c r="C86" s="25" t="inlineStr">
-        <is>
-          <t>A organização documenta procedimento para determinar coleta e análise de dados referente a reclamações, feedbacks, requisitos regulatórios, fornecedores, auditorias, relatórios de serviços e tratá-los?</t>
-        </is>
-      </c>
-      <c r="D86" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E86" s="27" t="n"/>
-      <c r="F86" s="27" t="n"/>
-      <c r="G86" s="27" t="n"/>
-      <c r="H86" s="35" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: PSQ.018.R2 - Realização de Produto; 
-PSQ.017.R3 - Controle de Documentos e Registros; 
-PSQ.019.R2 - Preservação de Insumo e Produto; 
-PSQ.022.R5 - Não Conformidade -Ações Corretivas e Preventivas; 
-PSQ.023.R4 - Treinamentos; 
-PSQ.024.R3 - Auditoria; 
-PSQ.026.R1 - Identificação e Rastreabilidade; 
-PSQ.027.R2 - Validação; 
-PSQ.028.R5 - Gestão de Risco; 
-PSQ.029.R3 - Gestão de Mudança; 
-PSQ.031.R0 - Gerenciamento de Claim de Produtos e Serviços; 
-PSQ.032.R7 - Monitoramento de Equipamento de Medição; 
-PSQ.033.R2 - Manutenção; 
-PSQ.025.R1 - Revisão Gerencial; 
-POP.1002.R1 - Manual Operacional - Rastreabilidade de Pedidos Visolab</t>
-        </is>
-      </c>
-      <c r="I86" s="35" t="n"/>
-      <c r="J86" s="128" t="n"/>
-      <c r="K86" s="22" t="n"/>
-      <c r="L86" s="22" t="n"/>
-      <c r="M86" s="22" t="n"/>
-    </row>
-    <row r="87" ht="96" customHeight="1" s="104">
-      <c r="A87" s="24" t="n"/>
-      <c r="B87" s="17" t="inlineStr">
-        <is>
-          <t>8.5.1</t>
-        </is>
-      </c>
-      <c r="C87" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A organização identifica e implementa ações para assegurar melhoria contínua do SGQ e outros processos relacionados ao produto? </t>
-        </is>
-      </c>
-      <c r="D87" s="28" t="n"/>
-      <c r="E87" s="27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F87" s="27" t="n"/>
-      <c r="G87" s="27" t="n"/>
-      <c r="H87" s="35" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: PSQ.018.R2 - Realização de Produto; 
-PSQ.017.R3 - Controle de Documentos e Registros; 
-PSQ.019.R2 - Preservação de Insumo e Produto; 
-PSQ.022.R5 - Não Conformidade -Ações Corretivas e Preventivas; 
-PSQ.023.R4 - Treinamentos; 
-PSQ.024.R3 - Auditoria; 
-PSQ.026.R1 - Identificação e Rastreabilidade; 
-PSQ.027.R2 - Validação; 
-PSQ.028.R5 - Gestão de Risco; 
-PSQ.029.R3 - Gestão de Mudança; 
-PSQ.031.R0 - Gerenciamento de Claim de Produtos e Serviços; 
-PSQ.032.R7 - Monitoramento de Equipamento de Medição; 
-PSQ.033.R2 - Manutenção; 
-PSQ.025.R1 - Revisão Gerencial; 
-POP.1002.R1 - Manual Operacional - Rastreabilidade de Pedidos Visolab
-• [Não Conforme] KPI - SERVICE RATE: Service Rate - Meta &gt;=95% - Nível de entrega no prazo
-Resultado: Não Conforme
-Realizado:  (Maio - 97,06%) (Junho -  91,17%) ( Julho - 96.88%)
-• [Não Conforme] KPI - LATE ORDERS: Meta &lt;=2,00% - Entrega de serviços em atraso com até 2 dias após o prazo
-Realizado:  (Maio - 0,86%) (Junho -  4,32%) ( Julho - 1,18%)</t>
-        </is>
-      </c>
-      <c r="I87" s="35" t="n"/>
-      <c r="J87" s="128" t="n"/>
-      <c r="K87" s="22" t="n"/>
-      <c r="L87" s="22" t="n"/>
-      <c r="M87" s="22" t="n"/>
-    </row>
-    <row r="88" ht="96" customHeight="1" s="104">
-      <c r="A88" s="24" t="n"/>
-      <c r="B88" s="17" t="inlineStr">
-        <is>
-          <t>8.5.2</t>
-        </is>
-      </c>
-      <c r="C88" s="25" t="inlineStr">
-        <is>
-          <t>A organização possui procedimento para ações corretivas que aborde a análise das não conformidades, avalia a necessidade de ações para que elas não recorram, necessidade de atualização de documentação e analise eficácia da ação adotada?</t>
-        </is>
-      </c>
-      <c r="D88" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E88" s="27" t="n"/>
-      <c r="F88" s="27" t="n"/>
-      <c r="G88" s="27" t="n"/>
-      <c r="H88" s="35" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: PSQ.018.R2 - Realização de Produto; 
-PSQ.017.R3 - Controle de Documentos e Registros; 
-PSQ.019.R2 - Preservação de Insumo e Produto; 
-PSQ.022.R5 - Não Conformidade -Ações Corretivas e Preventivas; 
-PSQ.023.R4 - Treinamentos; 
-PSQ.024.R3 - Auditoria; 
-PSQ.026.R1 - Identificação e Rastreabilidade; 
-PSQ.027.R2 - Validação; 
-PSQ.028.R5 - Gestão de Risco; 
-PSQ.029.R3 - Gestão de Mudança; 
-PSQ.031.R0 - Gerenciamento de Claim de Produtos e Serviços; 
-PSQ.032.R7 - Monitoramento de Equipamento de Medição; 
-PSQ.033.R2 - Manutenção; 
-PSQ.025.R1 - Revisão Gerencial; 
-POP.1002.R1 - Manual Operacional - Rastreabilidade de Pedidos Visolab</t>
-        </is>
-      </c>
-      <c r="I88" s="35" t="n"/>
-      <c r="J88" s="128" t="n"/>
-      <c r="K88" s="22" t="n"/>
-      <c r="L88" s="22" t="n"/>
-      <c r="M88" s="22" t="n"/>
-    </row>
-    <row r="89" ht="96" customHeight="1" s="104">
-      <c r="A89" s="24" t="n"/>
-      <c r="B89" s="17" t="inlineStr">
-        <is>
-          <t>8.5.3</t>
-        </is>
-      </c>
-      <c r="C89" s="25" t="inlineStr">
-        <is>
-          <t>A organização determina ações para eliminar causas de não conformidades potênciais? Possui procedimento para para determinação de não conformidades potenciais, avalia a necessidade de ações para prevenir novas não conformidades, planeja e documenta ações necessárias e as implementa conforme apropriado?</t>
-        </is>
-      </c>
-      <c r="D89" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E89" s="27" t="n"/>
-      <c r="F89" s="27" t="n"/>
-      <c r="G89" s="27" t="n"/>
-      <c r="H89" s="35" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: PSQ.018.R2 - Realização de Produto; 
-PSQ.017.R3 - Controle de Documentos e Registros; 
-PSQ.019.R2 - Preservação de Insumo e Produto; 
-PSQ.022.R5 - Não Conformidade -Ações Corretivas e Preventivas; 
-PSQ.023.R4 - Treinamentos; 
-PSQ.024.R3 - Auditoria; 
-PSQ.026.R1 - Identificação e Rastreabilidade; 
-PSQ.027.R2 - Validação; 
-PSQ.028.R5 - Gestão de Risco; 
-PSQ.029.R3 - Gestão de Mudança; 
-PSQ.031.R0 - Gerenciamento de Claim de Produtos e Serviços; 
-PSQ.032.R7 - Monitoramento de Equipamento de Medição; 
-PSQ.033.R2 - Manutenção; 
-PSQ.025.R1 - Revisão Gerencial; 
-POP.1002.R1 - Manual Operacional - Rastreabilidade de Pedidos Visolab</t>
-        </is>
-      </c>
-      <c r="I89" s="35" t="n"/>
-      <c r="J89" s="128" t="n"/>
-      <c r="K89" s="22" t="n"/>
-      <c r="L89" s="22" t="n"/>
-      <c r="M89" s="22" t="n"/>
-    </row>
-    <row r="90" ht="15.75" customHeight="1" s="104">
-      <c r="A90" s="5" t="n"/>
-      <c r="B90" s="7" t="n"/>
-      <c r="C90" s="38" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D90" s="153" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E90" s="154" t="n"/>
-      <c r="F90" s="155" t="n"/>
-      <c r="G90" s="156" t="n"/>
-      <c r="H90" s="157" t="inlineStr">
-        <is>
-          <t>• [Conforme] PSQ.022.R5: Não Conformidade - Ações Corretivas e Preventivas: A organização deve realizar o acompanhamento de todas as soluções de problemas e oportunidades de melhorias criadas para que o sistema de qualidade esteja em constante melhoria dos seus processos. Neste sentido, é obrigatório inserir todos os registros relacionados no Controle Anual de Registros: Plano de Ação, RNC, 8D, Gestão de Mudança e Revisão Gerencial.
-• [Conforme] POP.1057.R0: Manual Operacional - Comunicação com o Cliente - Visolab: 2. RECLAMAÇÕES: 
-2.1 Recebimento de Reclamações 
-2.2 Tratativa das Reclamações:
-3.DEVOLUTIVAS PARA O CLIENTE:
-As devolutivas aos clientes são enviadas de acordo com o canal utilizado pelo mesmo.
-• [Conforme] POP.1012.R1: Monitoramento de Realimentação do Cliente - Visolab: 2. REGISTRO DAS RECLAMAÇÕES DE CLIENTES:
-2.1 Registro de Realimentação de clientes através do atendimento
-3. ACOMPANHAMENTO DE RETORNOS:
-4. PESQUISA ANUAL DE SATISFAÇÃO</t>
-        </is>
-      </c>
-      <c r="I90" s="158" t="n"/>
-      <c r="J90" s="159" t="n"/>
-      <c r="K90" s="5" t="n"/>
-      <c r="L90" s="5" t="n"/>
-      <c r="M90" s="5" t="n"/>
-    </row>
-    <row r="91" ht="15.75" customHeight="1" s="104">
-      <c r="A91" s="5" t="n"/>
-      <c r="B91" s="7" t="n"/>
-      <c r="C91" s="38" t="inlineStr">
-        <is>
-          <t>NC</t>
-        </is>
-      </c>
-      <c r="D91" s="153" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E91" s="154" t="n"/>
-      <c r="F91" s="155" t="n"/>
-      <c r="G91" s="156" t="n"/>
-      <c r="H91" s="157" t="inlineStr">
-        <is>
-          <t>• [Conforme] PSQ.024.R3: Auditoria: FOR.140: Relatório de Auditoria Interna, 
-FOR.123: Agenda de Auditoria, 
-FOR.167: Cronograma de Auditoria, 
-FOR.143: Formulário de Check List da Auditoria ISO 1348</t>
-        </is>
-      </c>
-      <c r="I91" s="158" t="n"/>
-      <c r="J91" s="159" t="n"/>
-      <c r="K91" s="5" t="n"/>
-      <c r="L91" s="5" t="n"/>
-      <c r="M91" s="5" t="n"/>
-    </row>
-    <row r="92" ht="15.75" customHeight="1" s="104">
-      <c r="A92" s="5" t="n"/>
-      <c r="B92" s="7" t="n"/>
-      <c r="C92" s="38" t="inlineStr">
-        <is>
-          <t>OM</t>
-        </is>
-      </c>
-      <c r="D92" s="153" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E92" s="154" t="n"/>
-      <c r="F92" s="155" t="n"/>
-      <c r="G92" s="156" t="n"/>
-      <c r="H92" s="157" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: MAQ.002.R10 - Manual da Qualidade:
-- Objetivos da Qualidade</t>
-        </is>
-      </c>
-      <c r="I92" s="158" t="n"/>
-      <c r="J92" s="159" t="n"/>
-      <c r="K92" s="5" t="n"/>
-      <c r="L92" s="5" t="n"/>
-      <c r="M92" s="5" t="n"/>
-    </row>
-    <row r="93" ht="15.75" customHeight="1" s="104">
-      <c r="A93" s="5" t="n"/>
-      <c r="B93" s="7" t="n"/>
-      <c r="C93" s="38" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="D93" s="153" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E93" s="154" t="n"/>
-      <c r="F93" s="155" t="n"/>
-      <c r="G93" s="156" t="n"/>
-      <c r="H93" s="157" t="inlineStr">
-        <is>
-          <t>• [Conforme] Evidências / Documentos Registrados: PSQ.018.R2 - Realização de Produto; 
-PSQ.017.R3 - Controle de Documentos e Registros; 
-PSQ.019.R2 - Preservação de Insumo e Produto; 
-PSQ.022.R5 - Não Conformidade -Ações Corretivas e Preventivas; 
-PSQ.023.R4 - Treinamentos; 
-PSQ.024.R3 - Auditoria; 
-PSQ.026.R1 - Identificação e Rastreabilidade; 
-PSQ.027.R2 - Validação; 
-PSQ.028.R5 - Gestão de Risco; 
-PSQ.029.R3 - Gestão de Mudança; 
-PSQ.031.R0 - Gerenciamento de Claim de Produtos e Serviços; 
-PSQ.032.R7 - Monitoramento de Equipamento de Medição; 
-PSQ.033.R2 - Manutenção; 
-PSQ.025.R1 - Revisão Gerencial; 
-POP.1002.R1 - Manual Operacional - Rastreabilidade de Pedidos Visolab</t>
-        </is>
-      </c>
-      <c r="I93" s="158" t="n"/>
-      <c r="J93" s="159" t="n"/>
+      <c r="I93" s="145" t="n"/>
       <c r="K93" s="5" t="n"/>
       <c r="L93" s="5" t="n"/>
       <c r="M93" s="5" t="n"/>
@@ -4816,7 +4645,7 @@
       <c r="M94" s="5" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="92">
+  <mergeCells count="88">
     <mergeCell ref="I81:J81"/>
     <mergeCell ref="I89:J89"/>
     <mergeCell ref="B13:J13"/>
@@ -4881,23 +4710,19 @@
     <mergeCell ref="I50:J50"/>
     <mergeCell ref="I65:J65"/>
     <mergeCell ref="I34:J34"/>
-    <mergeCell ref="I90:J90"/>
     <mergeCell ref="I49:J49"/>
     <mergeCell ref="I27:J27"/>
     <mergeCell ref="I36:J36"/>
-    <mergeCell ref="I91:J91"/>
     <mergeCell ref="I85:J85"/>
     <mergeCell ref="B10:J10"/>
     <mergeCell ref="I75:J75"/>
     <mergeCell ref="I53:J53"/>
     <mergeCell ref="I22:J22"/>
     <mergeCell ref="I28:J28"/>
-    <mergeCell ref="I93:J93"/>
     <mergeCell ref="B74:J74"/>
     <mergeCell ref="C7:H7"/>
     <mergeCell ref="I12:J12"/>
     <mergeCell ref="I68:J68"/>
-    <mergeCell ref="I92:J92"/>
     <mergeCell ref="I55:J55"/>
     <mergeCell ref="I67:J67"/>
     <mergeCell ref="I5:J5"/>
@@ -9749,7 +9574,7 @@
         <f>H4</f>
         <v/>
       </c>
-      <c r="E44" s="137" t="n"/>
+      <c r="E44" s="146" t="n"/>
       <c r="F44" s="127" t="n"/>
       <c r="G44" s="127" t="n"/>
       <c r="H44" s="127" t="n"/>
@@ -9793,7 +9618,7 @@
         <f>H5</f>
         <v/>
       </c>
-      <c r="E45" s="138" t="n"/>
+      <c r="E45" s="147" t="n"/>
       <c r="F45" s="127" t="n"/>
       <c r="G45" s="127" t="n"/>
       <c r="H45" s="127" t="n"/>
@@ -9837,7 +9662,7 @@
         <f>H6</f>
         <v/>
       </c>
-      <c r="E46" s="138" t="n"/>
+      <c r="E46" s="147" t="n"/>
       <c r="F46" s="127" t="n"/>
       <c r="G46" s="127" t="n"/>
       <c r="H46" s="127" t="n"/>
@@ -9881,7 +9706,7 @@
         <f>H7</f>
         <v/>
       </c>
-      <c r="E47" s="138" t="n"/>
+      <c r="E47" s="147" t="n"/>
       <c r="F47" s="127" t="n"/>
       <c r="G47" s="127" t="n"/>
       <c r="H47" s="127" t="n"/>
@@ -9925,7 +9750,7 @@
         <f>H8</f>
         <v/>
       </c>
-      <c r="E48" s="138" t="n"/>
+      <c r="E48" s="147" t="n"/>
       <c r="F48" s="127" t="n"/>
       <c r="G48" s="127" t="n"/>
       <c r="H48" s="127" t="n"/>
@@ -42492,7 +42317,7 @@
 (Software utilizados desde o início do laboratório, garantindo sua eficiência e rastreabilidade. Caso ocorra alguma mudança, será validado no FOR.137)</t>
         </is>
       </c>
-      <c r="J3" s="139" t="inlineStr">
+      <c r="J3" s="148" t="inlineStr">
         <is>
           <t>Corporativo: Atualizar PSQ.027 - Procedimento de Validação. Criar formulários de validação de software.
 Corporativo + Rio: Preencher formulários de validação dos softwares (DECIDE, SMR, SGO, Optifacts e Qualiex).</t>
@@ -42505,7 +42330,7 @@
     </row>
     <row r="4" ht="63" customHeight="1" s="104">
       <c r="A4" s="24" t="n"/>
-      <c r="B4" s="140" t="inlineStr">
+      <c r="B4" s="149" t="inlineStr">
         <is>
           <t xml:space="preserve">RESPONSABILIDADE DA DIREÇÃO								</t>
         </is>
@@ -42555,7 +42380,7 @@
     </row>
     <row r="5" ht="37.8" customHeight="1" s="104">
       <c r="A5" s="24" t="n"/>
-      <c r="B5" s="141" t="n"/>
+      <c r="B5" s="150" t="n"/>
       <c r="C5" s="17" t="inlineStr">
         <is>
           <t>5.2</t>
@@ -42591,7 +42416,7 @@
     </row>
     <row r="6" ht="96" customHeight="1" s="104">
       <c r="A6" s="24" t="n"/>
-      <c r="B6" s="141" t="n"/>
+      <c r="B6" s="150" t="n"/>
       <c r="C6" s="17" t="inlineStr">
         <is>
           <t>5.5.1</t>
@@ -42633,7 +42458,7 @@
     </row>
     <row r="7" ht="37.8" customHeight="1" s="104">
       <c r="A7" s="24" t="n"/>
-      <c r="B7" s="141" t="n"/>
+      <c r="B7" s="150" t="n"/>
       <c r="C7" s="17" t="inlineStr">
         <is>
           <t>5.5.3</t>
@@ -42669,7 +42494,7 @@
     </row>
     <row r="8" ht="96" customHeight="1" s="104">
       <c r="A8" s="24" t="n"/>
-      <c r="B8" s="142" t="n"/>
+      <c r="B8" s="151" t="n"/>
       <c r="C8" s="17" t="inlineStr">
         <is>
           <t>5.6.3</t>
@@ -42708,7 +42533,7 @@
     </row>
     <row r="9" ht="138.6" customHeight="1" s="104">
       <c r="A9" s="24" t="n"/>
-      <c r="B9" s="140" t="inlineStr">
+      <c r="B9" s="149" t="inlineStr">
         <is>
           <t>GESTÃO DE RECURSOS</t>
         </is>
@@ -42756,7 +42581,7 @@
     </row>
     <row r="10" ht="153.75" customHeight="1" s="104">
       <c r="A10" s="24" t="n"/>
-      <c r="B10" s="142" t="n"/>
+      <c r="B10" s="151" t="n"/>
       <c r="C10" s="31" t="n">
         <v>44626</v>
       </c>
@@ -42780,7 +42605,7 @@
 **ver na aba evidências</t>
         </is>
       </c>
-      <c r="J10" s="143" t="inlineStr">
+      <c r="J10" s="152" t="inlineStr">
         <is>
           <t>Relatório para verificação das particulas da sala limpa não traz informações suficientes para comparar com o padrão.
 Será abordado na nova revisão gerencial para tomar novas ações para validação
@@ -42796,7 +42621,7 @@
     </row>
     <row r="11" ht="106.5" customHeight="1" s="104">
       <c r="A11" s="24" t="n"/>
-      <c r="B11" s="140" t="inlineStr">
+      <c r="B11" s="149" t="inlineStr">
         <is>
           <t xml:space="preserve">	REALIZAÇÃO DE PRODUTO (FABRICAÇÃO)</t>
         </is>
@@ -42846,7 +42671,7 @@
     </row>
     <row r="12" ht="88.2" customHeight="1" s="104">
       <c r="A12" s="24" t="n"/>
-      <c r="B12" s="141" t="n"/>
+      <c r="B12" s="150" t="n"/>
       <c r="C12" s="17" t="inlineStr">
         <is>
           <t>7.2.3</t>
@@ -42884,7 +42709,7 @@
     </row>
     <row r="13" ht="88.2" customHeight="1" s="104">
       <c r="A13" s="24" t="n"/>
-      <c r="B13" s="141" t="n"/>
+      <c r="B13" s="150" t="n"/>
       <c r="C13" s="17" t="inlineStr">
         <is>
           <t>7.5.1</t>
@@ -42924,7 +42749,7 @@
     </row>
     <row r="14" ht="96" customHeight="1" s="104">
       <c r="A14" s="24" t="n"/>
-      <c r="B14" s="141" t="n"/>
+      <c r="B14" s="150" t="n"/>
       <c r="C14" s="17" t="inlineStr">
         <is>
           <t>7.5.6</t>
@@ -42964,7 +42789,7 @@
     </row>
     <row r="15" ht="96" customHeight="1" s="104">
       <c r="A15" s="24" t="n"/>
-      <c r="B15" s="141" t="n"/>
+      <c r="B15" s="150" t="n"/>
       <c r="C15" s="17" t="inlineStr">
         <is>
           <t>7.5.8</t>
@@ -43000,7 +42825,7 @@
     </row>
     <row r="16" ht="96" customHeight="1" s="104">
       <c r="A16" s="24" t="n"/>
-      <c r="B16" s="141" t="n"/>
+      <c r="B16" s="150" t="n"/>
       <c r="C16" s="17" t="inlineStr">
         <is>
           <t>7.5.9.1</t>
@@ -43037,7 +42862,7 @@
     </row>
     <row r="17" ht="96" customHeight="1" s="104">
       <c r="A17" s="24" t="n"/>
-      <c r="B17" s="141" t="n"/>
+      <c r="B17" s="150" t="n"/>
       <c r="C17" s="17" t="inlineStr">
         <is>
           <t>7.5.10</t>
@@ -43074,7 +42899,7 @@
     </row>
     <row r="18" ht="201.6" customHeight="1" s="104">
       <c r="A18" s="24" t="n"/>
-      <c r="B18" s="141" t="n"/>
+      <c r="B18" s="150" t="n"/>
       <c r="C18" s="17" t="inlineStr">
         <is>
           <t>7.5.11</t>
@@ -43116,7 +42941,7 @@
     </row>
     <row r="19" ht="96" customHeight="1" s="104">
       <c r="A19" s="24" t="n"/>
-      <c r="B19" s="142" t="n"/>
+      <c r="B19" s="151" t="n"/>
       <c r="C19" s="17" t="inlineStr">
         <is>
           <t>7.6</t>
@@ -43152,7 +42977,7 @@
     </row>
     <row r="20" ht="96" customHeight="1" s="104">
       <c r="A20" s="24" t="n"/>
-      <c r="B20" s="140" t="inlineStr">
+      <c r="B20" s="149" t="inlineStr">
         <is>
           <t>MEDIÇÃO, ANÁLISE E MELHORIA</t>
         </is>
@@ -43201,7 +43026,7 @@
     </row>
     <row r="21" ht="96" customHeight="1" s="104">
       <c r="A21" s="24" t="n"/>
-      <c r="B21" s="141" t="n"/>
+      <c r="B21" s="150" t="n"/>
       <c r="C21" s="17" t="inlineStr">
         <is>
           <t>8.2.1</t>
@@ -43238,7 +43063,7 @@
     </row>
     <row r="22" ht="100.8" customHeight="1" s="104">
       <c r="A22" s="80" t="n"/>
-      <c r="B22" s="141" t="n"/>
+      <c r="B22" s="150" t="n"/>
       <c r="C22" s="81" t="inlineStr">
         <is>
           <t>8.2.2</t>
@@ -43277,7 +43102,7 @@
     </row>
     <row r="23" ht="113.4" customHeight="1" s="104">
       <c r="A23" s="80" t="n"/>
-      <c r="B23" s="141" t="n"/>
+      <c r="B23" s="150" t="n"/>
       <c r="C23" s="86" t="inlineStr">
         <is>
           <t>8.2.4</t>
@@ -43310,14 +43135,14 @@
 - LabRio: realizar tratativas dos resultados das auditorias</t>
         </is>
       </c>
-      <c r="K23" s="144" t="n"/>
+      <c r="K23" s="153" t="n"/>
       <c r="L23" s="85" t="n"/>
       <c r="M23" s="85" t="n"/>
       <c r="N23" s="85" t="n"/>
     </row>
     <row r="24" ht="96" customHeight="1" s="104">
       <c r="A24" s="24" t="n"/>
-      <c r="B24" s="141" t="n"/>
+      <c r="B24" s="150" t="n"/>
       <c r="C24" s="17" t="inlineStr">
         <is>
           <t>8.2.5</t>
@@ -43356,7 +43181,7 @@
     </row>
     <row r="25" ht="96" customHeight="1" s="104">
       <c r="A25" s="24" t="n"/>
-      <c r="B25" s="141" t="n"/>
+      <c r="B25" s="150" t="n"/>
       <c r="C25" s="17" t="inlineStr">
         <is>
           <t>8.2.6</t>
@@ -43394,7 +43219,7 @@
     </row>
     <row r="26" ht="88.2" customHeight="1" s="104">
       <c r="A26" s="24" t="n"/>
-      <c r="B26" s="141" t="n"/>
+      <c r="B26" s="150" t="n"/>
       <c r="C26" s="17" t="inlineStr">
         <is>
           <t>8.3.3</t>
@@ -43431,7 +43256,7 @@
     </row>
     <row r="27" ht="96" customHeight="1" s="104">
       <c r="A27" s="24" t="n"/>
-      <c r="B27" s="141" t="n"/>
+      <c r="B27" s="150" t="n"/>
       <c r="C27" s="17" t="inlineStr">
         <is>
           <t>8.4</t>
@@ -43469,7 +43294,7 @@
     </row>
     <row r="28" ht="96" customHeight="1" s="104">
       <c r="A28" s="24" t="n"/>
-      <c r="B28" s="141" t="n"/>
+      <c r="B28" s="150" t="n"/>
       <c r="C28" s="17" t="inlineStr">
         <is>
           <t>8.5.1</t>
@@ -43502,7 +43327,7 @@
     </row>
     <row r="29" ht="96" customHeight="1" s="104">
       <c r="A29" s="24" t="n"/>
-      <c r="B29" s="141" t="n"/>
+      <c r="B29" s="150" t="n"/>
       <c r="C29" s="17" t="inlineStr">
         <is>
           <t>8.5.2</t>
@@ -43539,7 +43364,7 @@
     </row>
     <row r="30" ht="96" customHeight="1" s="104">
       <c r="A30" s="24" t="n"/>
-      <c r="B30" s="142" t="n"/>
+      <c r="B30" s="151" t="n"/>
       <c r="C30" s="17" t="inlineStr">
         <is>
           <t>8.5.3</t>

</xml_diff>